<commit_message>
Rewrite Phase 0 as a from-scratch GenAI on-ramp
Replace the Staff/Principal-heavy 00-01 chapter with beginner-friendly
GenAI vocabulary, simple diagrams, and a Hello-LLM lab. Reorder Phase 0
to 00-01 → Python/APIs → Math, deferring BankCo/production drills until
after the first model call, and sync roadmap/study/dashboard/tracker.

Co-authored-by: Rahul Chaudhari <rcrahul4@gmail.com>
</commit_message>
<xml_diff>
--- a/Tracker/GenAI-Masterclass-Tracker.xlsx
+++ b/Tracker/GenAI-Masterclass-Tracker.xlsx
@@ -860,17 +860,17 @@
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>00-01, 00-02, 00-03</t>
+          <t>00-01, 00-05, 00-06, 00-04</t>
         </is>
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>BankCo decision agent</t>
+          <t>Hello-LLM CLI + FastAPI warmup</t>
         </is>
       </c>
       <c r="F2" s="11" t="inlineStr">
         <is>
-          <t>AI judgment</t>
+          <t>GenAI vocabulary</t>
         </is>
       </c>
       <c r="G2" s="11" t="n">
@@ -883,10 +883,10 @@
         </is>
       </c>
       <c r="J2" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K2" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-05",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-05",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-06",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-06",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-04",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L2" s="13">
@@ -5082,7 +5082,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>00-01 — AI Engineering Mindset for Principal, Staff &amp; Engineering Managers</t>
+          <t>00-01 — GenAI From Scratch: Core Ideas</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -8115,7 +8115,7 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>00-01 — AI Engineering Mindset for Principal, Staff &amp; Engineering Managers</t>
+          <t>00-01 — GenAI From Scratch: Core Ideas</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
@@ -8140,7 +8140,7 @@
         </is>
       </c>
       <c r="H2" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
@@ -11721,12 +11721,12 @@
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>LangGraph Overview</t>
+          <t>OpenAI — Text generation / chat concepts</t>
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr">
         <is>
-          <t>https://langchain-ai.github.io/langgraph/concepts/high_level/</t>
+          <t>https://platform.openai.com/docs/guides/text</t>
         </is>
       </c>
       <c r="G2" s="12">
@@ -11744,17 +11744,17 @@
       </c>
       <c r="J2" s="11" t="inlineStr">
         <is>
-          <t>20 min</t>
+          <t>20–30 min</t>
         </is>
       </c>
       <c r="K2" s="11" t="inlineStr">
         <is>
-          <t>See production agent runtime concerns (persistence, HITL)</t>
+          <t>Solidify messages, models, tokens</t>
         </is>
       </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>Core benefits; ecosystem; persistence</t>
+          <t>Messages; models; token basics</t>
         </is>
       </c>
       <c r="M2" s="11" t="inlineStr">
@@ -11790,12 +11790,12 @@
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>MCP Intro</t>
+          <t>Anthropic — Claude overview</t>
         </is>
       </c>
       <c r="F3" s="12" t="inlineStr">
         <is>
-          <t>https://modelcontextprotocol.io/docs/getting-started/intro</t>
+          <t>https://docs.anthropic.com/en/docs/welcome</t>
         </is>
       </c>
       <c r="G3" s="12">
@@ -11813,17 +11813,17 @@
       </c>
       <c r="J3" s="11" t="inlineStr">
         <is>
-          <t>15 min</t>
+          <t>20 min</t>
         </is>
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>Standard tool connectivity mindset</t>
+          <t>Second provider vocabulary</t>
         </is>
       </c>
       <c r="L3" s="11" t="inlineStr">
         <is>
-          <t>What MCP enables; why it matters</t>
+          <t>Messages API mental model</t>
         </is>
       </c>
       <c r="M3" s="11" t="inlineStr">
@@ -11859,12 +11859,12 @@
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>OpenAI Prompt Engineering Guide</t>
+          <t>Google — Gemini API quickstart</t>
         </is>
       </c>
       <c r="F4" s="12" t="inlineStr">
         <is>
-          <t>https://developers.openai.com/api/docs/guides/prompt-engineering</t>
+          <t>https://ai.google.dev/gemini-api/docs/quickstart</t>
         </is>
       </c>
       <c r="G4" s="12">
@@ -11882,17 +11882,17 @@
       </c>
       <c r="J4" s="11" t="inlineStr">
         <is>
-          <t>45 min</t>
+          <t>20 min</t>
         </is>
       </c>
       <c r="K4" s="11" t="inlineStr">
         <is>
-          <t>Prompt as contract, not poetry</t>
+          <t>Multi-provider habit early</t>
         </is>
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Tactics; message roles; iteration</t>
+          <t>First request</t>
         </is>
       </c>
       <c r="M4" s="11" t="inlineStr">
@@ -11928,12 +11928,12 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Anthropic / Claude Docs Overview</t>
+          <t>DeepSeek API docs</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>https://platform.claude.com/docs/en/docs/build-with-claude/overview</t>
+          <t>https://api-docs.deepseek.com/</t>
         </is>
       </c>
       <c r="G5" s="12">
@@ -11951,17 +11951,17 @@
       </c>
       <c r="J5" s="11" t="inlineStr">
         <is>
-          <t>30 min</t>
+          <t>15 min</t>
         </is>
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>Alternate provider constraints</t>
+          <t>Cost-efficient OpenAI-compatible option</t>
         </is>
       </c>
       <c r="L5" s="11" t="inlineStr">
         <is>
-          <t>Build with Claude overview</t>
+          <t>First chat call</t>
         </is>
       </c>
       <c r="M5" s="11" t="inlineStr">
@@ -11997,12 +11997,12 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Attention Is All You Need</t>
+          <t>OpenAI Prompt Engineering Guide</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/1706.03762</t>
+          <t>https://developers.openai.com/api/docs/guides/prompt-engineering</t>
         </is>
       </c>
       <c r="G6" s="12">
@@ -12015,22 +12015,22 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Intro</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
         <is>
-          <t>60–90 min</t>
+          <t>45 min</t>
         </is>
       </c>
       <c r="K6" s="11" t="inlineStr">
         <is>
-          <t>Shared vocabulary for later chapters</t>
+          <t>Prompts as clear instructions</t>
         </is>
       </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>Architecture diagram; attention</t>
+          <t>Tactics; iteration</t>
         </is>
       </c>
       <c r="M6" s="11" t="inlineStr">
@@ -12066,12 +12066,12 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>ReAct: Synergizing Reasoning and Acting</t>
+          <t>Chip Huyen — *AI Engineering* (book)</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2210.03629</t>
+          <t>https://www.oreilly.com/library/view/ai-engineering/9781098166298/</t>
         </is>
       </c>
       <c r="G7" s="12">
@@ -12089,17 +12089,17 @@
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>45 min</t>
+          <t>ongoing</t>
         </is>
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>Grounds the agent loop chapter</t>
+          <t>Bridge from ideas to production later</t>
         </is>
       </c>
       <c r="L7" s="11" t="inlineStr">
         <is>
-          <t>Think-Act-Observe examples</t>
+          <t>Early chapters on AI eng vs ML eng</t>
         </is>
       </c>
       <c r="M7" s="11" t="inlineStr">
@@ -12135,12 +12135,12 @@
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>OWASP Top 10 for LLM Applications</t>
+          <t>Karpathy — Intro to LLMs (talk)</t>
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>https://owasp.org/www-project-top-10-for-large-language-model-applications/</t>
+          <t>https://www.youtube.com/watch?v=zjkBMFhNj_g</t>
         </is>
       </c>
       <c r="G8" s="12">
@@ -12153,7 +12153,7 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Intro</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
@@ -12163,12 +12163,12 @@
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>Safety mindset early</t>
+          <t>Intuition without heavy math</t>
         </is>
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>LLM01 Prompt Injection; data leakage</t>
+          <t>Whole talk once</t>
         </is>
       </c>
       <c r="M8" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Align full curriculum sequencing after GenAI from-scratch on-ramp
Audit and fix navigation/prereq drift so beginners follow
00-01 → Python/APIs → Math → Rules/Agents before Staff+ chapters.
Schedule 00-02/00-03, correct Roadmap Day-1 CTA, Resource Database,
Architecture Index patterns, Career Q maps, broken Related links,
and rebuild the Excel tracker week/project mappings.

Co-authored-by: Rahul Chaudhari <rcrahul4@gmail.com>
</commit_message>
<xml_diff>
--- a/Tracker/GenAI-Masterclass-Tracker.xlsx
+++ b/Tracker/GenAI-Masterclass-Tracker.xlsx
@@ -28,9 +28,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Resources'!$A$1:$O$292</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'SystemDesign'!$A$1:$P$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'LeadershipCareer'!$A$1:$K$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Weekly'!$A$1:$M$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Weekly'!$A$1:$M$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'DailyLog'!$A$1:$N$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Projects'!$A$1:$M$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Projects'!$A$1:$M$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Interviews'!$A$1:$M$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'STAR'!$A$1:$N$9</definedName>
   </definedNames>
@@ -759,7 +759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -850,7 +850,7 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Foundations</t>
+          <t>Foundations — GenAI + craft</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
@@ -901,27 +901,27 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>LLM Engineering I</t>
+          <t>Foundations — Rules / BankCo</t>
         </is>
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>01 LLM Engineering</t>
+          <t>00 Foundations</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>01-01, 01-02</t>
+          <t>00-02, 00-03</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>Token cost estimator</t>
+          <t>When-not-to-agent memo · BankCo rules</t>
         </is>
       </c>
       <c r="F3" s="11" t="inlineStr">
         <is>
-          <t>Transformer whiteboard</t>
+          <t>Rules vs agent</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
@@ -937,7 +937,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"01-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"01-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-02",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L3" s="13">
@@ -952,7 +952,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>LLM Engineering II</t>
+          <t>LLM Engineering I</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
@@ -962,17 +962,17 @@
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>01-03, 01-04, 01-05</t>
+          <t>01-01, 01-02</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>LiteLLM FastAPI router</t>
+          <t>Token cost estimator</t>
         </is>
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>Inference tradeoffs</t>
+          <t>Transformer whiteboard</t>
         </is>
       </c>
       <c r="G4" s="11" t="n">
@@ -985,10 +985,10 @@
         </is>
       </c>
       <c r="J4" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K4" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"01-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"01-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-04",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"01-05",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-05",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"01-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"01-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-02",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L4" s="13">
@@ -1003,27 +1003,27 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Prompts &amp; Tools</t>
+          <t>LLM Engineering II</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>02 Prompt Engineering</t>
+          <t>01 LLM Engineering</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>02-01, 02-02</t>
+          <t>01-03, 01-04, 01-05</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Structured router agent</t>
+          <t>LiteLLM FastAPI router</t>
         </is>
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>Tool-calling design</t>
+          <t>Inference tradeoffs</t>
         </is>
       </c>
       <c r="G5" s="11" t="n">
@@ -1036,10 +1036,10 @@
         </is>
       </c>
       <c r="J5" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K5" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"02-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"02-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"02-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"02-02",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"01-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"01-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-04",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"01-05",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-05",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L5" s="13">
@@ -1054,27 +1054,27 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Agents I</t>
+          <t>Prompts &amp; Tools</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>03 Agentic Fundamentals</t>
+          <t>02 Prompt Engineering</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>03-01, 03-02</t>
+          <t>02-01, 02-02</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Inquiry routing agent</t>
+          <t>Structured router agent</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>Agent loop critique</t>
+          <t>Tool-calling design</t>
         </is>
       </c>
       <c r="G6" s="11" t="n">
@@ -1090,7 +1090,7 @@
         <v>2</v>
       </c>
       <c r="K6" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"03-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"03-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-02",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"02-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"02-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"02-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"02-02",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L6" s="13">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Agents II</t>
+          <t>Agents I</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -1115,17 +1115,17 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>03-03, 03-04</t>
+          <t>03-01, 03-02</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>LangGraph + checkpointing</t>
+          <t>Inquiry routing agent</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>Pattern selection</t>
+          <t>Agent loop critique</t>
         </is>
       </c>
       <c r="G7" s="11" t="n">
@@ -1141,7 +1141,7 @@
         <v>2</v>
       </c>
       <c r="K7" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"03-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"03-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-04",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"03-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"03-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-02",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L7" s="13">
@@ -1156,27 +1156,27 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>RAG I</t>
+          <t>Agents II</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>04 RAG</t>
+          <t>03 Agentic Fundamentals</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>04-01, 04-02</t>
+          <t>03-03, 03-04</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>Ingestion + chunking</t>
+          <t>LangGraph + checkpointing</t>
         </is>
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>Chunking tradeoffs</t>
+          <t>Pattern selection</t>
         </is>
       </c>
       <c r="G8" s="11" t="n">
@@ -1192,7 +1192,7 @@
         <v>2</v>
       </c>
       <c r="K8" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"04-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"04-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-02",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"03-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"03-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-04",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L8" s="13">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>RAG II</t>
+          <t>RAG I</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -1217,17 +1217,17 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>04-03, 04-04</t>
+          <t>04-01, 04-02</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Hybrid + rerank + citations</t>
+          <t>Ingestion + chunking</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Hallucination control</t>
+          <t>Chunking tradeoffs</t>
         </is>
       </c>
       <c r="G9" s="11" t="n">
@@ -1243,7 +1243,7 @@
         <v>2</v>
       </c>
       <c r="K9" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"04-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"04-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-04",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"04-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"04-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-02",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L9" s="13">
@@ -1258,31 +1258,31 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>RAG II</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>05 Multi-Agent</t>
+          <t>04 RAG</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>05-01, 05-02, 05-03</t>
+          <t>04-03, 04-04</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Travel planner multi-agent</t>
+          <t>Hybrid + rerank + citations</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>Coordination failures</t>
+          <t>Hallucination control</t>
         </is>
       </c>
       <c r="G10" s="11" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H10" s="11" t="inlineStr"/>
       <c r="I10" s="11" t="inlineStr">
@@ -1291,10 +1291,10 @@
         </is>
       </c>
       <c r="J10" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K10" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"05-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"05-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"05-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"05-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"05-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"05-03",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"04-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"04-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-04",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L10" s="13">
@@ -1309,31 +1309,31 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Voice / Multimodal</t>
+          <t>Multi-Agent</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>06 Voice &amp; Multimodal</t>
+          <t>05 Multi-Agent</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>06-01, 06-02</t>
+          <t>05-01, 05-02, 05-03</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>ASR→LLM→TTS bot</t>
+          <t>Travel planner multi-agent</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>Latency budgets</t>
+          <t>Coordination failures</t>
         </is>
       </c>
       <c r="G11" s="11" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H11" s="11" t="inlineStr"/>
       <c r="I11" s="11" t="inlineStr">
@@ -1342,10 +1342,10 @@
         </is>
       </c>
       <c r="J11" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K11" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"06-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"06-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"06-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"06-02",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"05-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"05-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"05-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"05-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"05-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"05-03",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L11" s="13">
@@ -1360,27 +1360,27 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Protocols</t>
+          <t>Voice / Multimodal</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>07 Protocols MCP/A2A</t>
+          <t>06 Voice &amp; Multimodal</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>07-01, 07-02, 07-03</t>
+          <t>06-01, 06-02</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>MCP + A2A negotiation</t>
+          <t>ASR→LLM→TTS bot</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>Protocol design</t>
+          <t>Latency budgets</t>
         </is>
       </c>
       <c r="G12" s="11" t="n">
@@ -1393,10 +1393,10 @@
         </is>
       </c>
       <c r="J12" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K12" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"07-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"07-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"07-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"07-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"07-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"07-03",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"06-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"06-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"06-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"06-02",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L12" s="13">
@@ -1411,27 +1411,27 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Eval / LLMOps</t>
+          <t>Protocols</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>08 Eval &amp; LLMOps</t>
+          <t>07 Protocols MCP/A2A</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>08-01, 08-02, 08-03</t>
+          <t>07-01, 07-02, 07-03, 07-04</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Golden set + ship gate</t>
+          <t>MCP + A2A negotiation</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>Eval strategy</t>
+          <t>Protocol design</t>
         </is>
       </c>
       <c r="G13" s="11" t="n">
@@ -1444,10 +1444,10 @@
         </is>
       </c>
       <c r="J13" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"08-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"08-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"08-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"08-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"08-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"08-03",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"07-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"07-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"07-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"07-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"07-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"07-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"07-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"07-04",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L13" s="13">
@@ -1462,27 +1462,27 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Fine-Tuning</t>
+          <t>Eval / LLMOps</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>09 Fine-Tuning</t>
+          <t>08 Eval &amp; LLMOps</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>09-01, 09-02, 09-03</t>
+          <t>08-01, 08-02, 08-03</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>LoRA compare</t>
+          <t>Golden set + ship gate</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>Prompt vs RAG vs FT</t>
+          <t>Eval strategy</t>
         </is>
       </c>
       <c r="G14" s="11" t="n">
@@ -1498,7 +1498,7 @@
         <v>3</v>
       </c>
       <c r="K14" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"09-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"09-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"09-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"09-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"09-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"09-03",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"08-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"08-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"08-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"08-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"08-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"08-03",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L14" s="13">
@@ -1513,31 +1513,31 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Production Infra</t>
+          <t>Fine-Tuning</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>10 Production Infra</t>
+          <t>09 Fine-Tuning</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>10-01, 10-02, 10-03, 10-04</t>
+          <t>09-01, 09-02, 09-03</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>Dockerized agent API</t>
+          <t>LoRA compare</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>Cost/latency design</t>
+          <t>Prompt vs RAG vs FT</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H15" s="11" t="inlineStr"/>
       <c r="I15" s="11" t="inlineStr">
@@ -1546,10 +1546,10 @@
         </is>
       </c>
       <c r="J15" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K15" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"10-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"10-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"10-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"10-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-04",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"09-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"09-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"09-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"09-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"09-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"09-03",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L15" s="13">
@@ -1564,27 +1564,27 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Security + Advanced</t>
+          <t>Production Infra</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>11 Security &amp; Safety</t>
+          <t>10 Production Infra</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>11-01, 11-02, 12-01, 12-02</t>
+          <t>10-01, 10-02, 10-03, 10-04</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Red-team + Text2SQL</t>
+          <t>Dockerized agent API</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Safety review</t>
+          <t>Cost/latency design</t>
         </is>
       </c>
       <c r="G16" s="11" t="n">
@@ -1600,7 +1600,7 @@
         <v>4</v>
       </c>
       <c r="K16" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"11-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"11-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"11-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"11-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-02",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"10-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"10-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"10-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"10-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-04",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L16" s="13">
@@ -1615,27 +1615,27 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Advanced + Capstone</t>
+          <t>Security + Advanced</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>12 Advanced Topics</t>
+          <t>11 Security &amp; Safety</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>12-03, 12-04</t>
+          <t>11-01, 11-02, 12-01, 12-02</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>Capstone vertical slice</t>
+          <t>Red-team + Text2SQL</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>Full design interview</t>
+          <t>Safety review</t>
         </is>
       </c>
       <c r="G17" s="11" t="n">
@@ -1648,10 +1648,10 @@
         </is>
       </c>
       <c r="J17" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K17" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"12-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-04",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"11-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"11-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"11-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"11-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-02",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L17" s="13">
@@ -1666,31 +1666,31 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Capstone + Mocks</t>
+          <t>Advanced + Capstone</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Capstone</t>
+          <t>12 Advanced Topics</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>CAPSTONE</t>
+          <t>12-03, 12-04, 12-05, 12-06</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Capstone v1 + 4 mocks</t>
+          <t>Capstone vertical slice</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>Panel simulation</t>
+          <t>Full design interview</t>
         </is>
       </c>
       <c r="G18" s="11" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H18" s="11" t="inlineStr"/>
       <c r="I18" s="11" t="inlineStr">
@@ -1699,10 +1699,10 @@
         </is>
       </c>
       <c r="J18" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K18" s="11">
-        <f>COUNTIFS(Projects!D:D,"Capstone",Projects!F:F,"Done")+COUNTIFS(Projects!D:D,"Capstone",Projects!F:F,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"12-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-04",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-05",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-05",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-06",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-06",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L18" s="13">
@@ -1711,10 +1711,61 @@
       </c>
       <c r="M18" s="11" t="n"/>
     </row>
+    <row r="19">
+      <c r="A19" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Capstone + Mocks</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Capstone</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>CAPSTONE</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Capstone v1 + 4 mocks</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Panel simulation</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="H19" s="11" t="inlineStr"/>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="11">
+        <f>COUNTIFS(Projects!D:D,"Capstone",Projects!F:F,"Done")+COUNTIFS(Projects!D:D,"Capstone",Projects!F:F,"Interview-ready")</f>
+        <v/>
+      </c>
+      <c r="L19" s="13">
+        <f>IF(J19=0,"",K19/J19)</f>
+        <v/>
+      </c>
+      <c r="M19" s="11" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M18"/>
+  <autoFilter ref="A1:M19"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Done,Interview-ready"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3289,7 +3340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3382,7 +3433,7 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>BankCo Decision Support</t>
+          <t>Hello-LLM Explain-It Bot</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
@@ -3405,7 +3456,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>00-01, 00-03</t>
+          <t>00-01</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr"/>
@@ -3434,17 +3485,17 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>P01b</t>
         </is>
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>Token Cost Estimator</t>
+          <t>BankCo Decision Support</t>
         </is>
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>LLM Projects</t>
+          <t>Foundations Projects</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
@@ -3462,7 +3513,7 @@
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
-          <t>01-02</t>
+          <t>00-02, 00-03</t>
         </is>
       </c>
       <c r="H3" s="11" t="inlineStr"/>
@@ -3491,12 +3542,12 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>LiteLLM Gateway</t>
+          <t>Token Cost Estimator</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
@@ -3519,7 +3570,7 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>01-04, 01-05</t>
+          <t>01-02</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr"/>
@@ -3548,22 +3599,22 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>P03</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Structured Router Agent</t>
+          <t>LiteLLM Gateway</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Agent Projects</t>
+          <t>LLM Projects</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Mini</t>
         </is>
       </c>
       <c r="E5" s="11" t="n">
@@ -3576,7 +3627,7 @@
       </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
-          <t>02-02, 03-03</t>
+          <t>01-04, 01-05</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr"/>
@@ -3605,12 +3656,12 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Inquiry Routing Agent</t>
+          <t>Structured Router Agent</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -3633,7 +3684,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>03-01, 03-02</t>
+          <t>02-02, 03-03</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr"/>
@@ -3662,12 +3713,12 @@
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>P06</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>LangGraph Production Agent</t>
+          <t>Inquiry Routing Agent</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -3690,7 +3741,7 @@
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
-          <t>03-04</t>
+          <t>03-01, 03-02</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr"/>
@@ -3719,26 +3770,26 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>P06</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>NovaCart RAG Assistant</t>
+          <t>LangGraph Production Agent</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>RAG Projects</t>
+          <t>Agent Projects</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="E8" s="11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
@@ -3747,7 +3798,7 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>04-01, 04-02, 04-03</t>
+          <t>03-04</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr"/>
@@ -3776,17 +3827,17 @@
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Multi-Agent Travel Planner</t>
+          <t>NovaCart RAG Assistant</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Multi-Agent Projects</t>
+          <t>RAG Projects</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
@@ -3804,7 +3855,7 @@
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>05-01, 05-02</t>
+          <t>04-01, 04-02, 04-03</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr"/>
@@ -3833,22 +3884,22 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Voice Bot</t>
+          <t>Multi-Agent Travel Planner</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Multimodal Projects</t>
+          <t>Multi-Agent Projects</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
@@ -3861,7 +3912,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>06-01</t>
+          <t>05-01, 05-02</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr"/>
@@ -3890,22 +3941,22 @@
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>MCP + Negotiation Sim</t>
+          <t>Voice Bot</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Protocol Projects</t>
+          <t>Multimodal Projects</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
@@ -3918,7 +3969,7 @@
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>07-01, 07-02, 07-03</t>
+          <t>06-01</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr"/>
@@ -3947,17 +3998,17 @@
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Eval Harness + Ship Gate</t>
+          <t>MCP + Negotiation Sim</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>LLMOps Projects</t>
+          <t>Protocol Projects</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -3975,7 +4026,7 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>08-01, 08-03</t>
+          <t>07-01, 07-02, 07-03</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr"/>
@@ -4004,22 +4055,22 @@
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>LoRA Integration</t>
+          <t>Eval Harness + Ship Gate</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Fine-Tune Projects</t>
+          <t>LLMOps Projects</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="E13" s="11" t="n">
@@ -4032,7 +4083,7 @@
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>09-01, 09-02, 09-03</t>
+          <t>08-01, 08-03</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr"/>
@@ -4061,22 +4112,22 @@
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Deployed Agent API</t>
+          <t>LoRA Integration</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Infra Projects</t>
+          <t>Fine-Tune Projects</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="E14" s="11" t="n">
@@ -4089,7 +4140,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>10-01, 10-02, 10-04</t>
+          <t>09-01, 09-02, 09-03</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr"/>
@@ -4118,26 +4169,26 @@
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Capstone Multi-Agent System</t>
+          <t>Deployed Agent API</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Capstone</t>
+          <t>Infra Projects</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Capstone</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
@@ -4146,7 +4197,7 @@
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>05-01, 04-01, 08-01, 11-01</t>
+          <t>10-01, 10-02, 10-04</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr"/>
@@ -4172,9 +4223,66 @@
       </c>
       <c r="M15" s="11" t="inlineStr"/>
     </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Capstone Multi-Agent System</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Capstone</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Capstone</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>05-01, 04-01, 08-01, 11-01</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr"/>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K16" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L16" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M16" s="11" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M15"/>
-  <conditionalFormatting sqref="F2:F15">
+  <autoFilter ref="A1:M16"/>
+  <conditionalFormatting sqref="F2:F16">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F2="Done"</formula>
     </cfRule>
@@ -4183,22 +4291,22 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
-    <dataValidation sqref="F2:F15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Done,Interview-ready"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Mini,Intermediate,Production,Capstone"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4699,7 +4807,7 @@
       <c r="G2" s="11" t="inlineStr"/>
       <c r="H2" s="11" t="inlineStr">
         <is>
-          <t>00-01, 08-03</t>
+          <t>12-06, 08-03</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr"/>
@@ -4963,7 +5071,7 @@
       <c r="G8" s="11" t="inlineStr"/>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>00-01</t>
+          <t>12-06</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr"/>
@@ -5123,7 +5231,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <f>IFERROR(VLOOKUP(A3,Modules!$A:$I,9,FALSE),"")</f>
@@ -5155,7 +5263,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <f>IFERROR(VLOOKUP(A4,Modules!$A:$I,9,FALSE),"")</f>
@@ -5283,7 +5391,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8">
         <f>IFERROR(VLOOKUP(A8,Modules!$A:$I,9,FALSE),"")</f>
@@ -5315,7 +5423,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9">
         <f>IFERROR(VLOOKUP(A9,Modules!$A:$I,9,FALSE),"")</f>
@@ -5347,7 +5455,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10">
         <f>IFERROR(VLOOKUP(A10,Modules!$A:$I,9,FALSE),"")</f>
@@ -5379,7 +5487,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11">
         <f>IFERROR(VLOOKUP(A11,Modules!$A:$I,9,FALSE),"")</f>
@@ -5411,7 +5519,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12">
         <f>IFERROR(VLOOKUP(A12,Modules!$A:$I,9,FALSE),"")</f>
@@ -5443,7 +5551,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E13">
         <f>IFERROR(VLOOKUP(A13,Modules!$A:$I,9,FALSE),"")</f>
@@ -5475,7 +5583,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E14">
         <f>IFERROR(VLOOKUP(A14,Modules!$A:$I,9,FALSE),"")</f>
@@ -5507,7 +5615,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E15">
         <f>IFERROR(VLOOKUP(A15,Modules!$A:$I,9,FALSE),"")</f>
@@ -5539,7 +5647,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E16">
         <f>IFERROR(VLOOKUP(A16,Modules!$A:$I,9,FALSE),"")</f>
@@ -5571,7 +5679,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E17">
         <f>IFERROR(VLOOKUP(A17,Modules!$A:$I,9,FALSE),"")</f>
@@ -5603,7 +5711,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E18">
         <f>IFERROR(VLOOKUP(A18,Modules!$A:$I,9,FALSE),"")</f>
@@ -5635,7 +5743,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E19">
         <f>IFERROR(VLOOKUP(A19,Modules!$A:$I,9,FALSE),"")</f>
@@ -5667,7 +5775,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E20">
         <f>IFERROR(VLOOKUP(A20,Modules!$A:$I,9,FALSE),"")</f>
@@ -5699,7 +5807,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E21">
         <f>IFERROR(VLOOKUP(A21,Modules!$A:$I,9,FALSE),"")</f>
@@ -5731,7 +5839,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E22">
         <f>IFERROR(VLOOKUP(A22,Modules!$A:$I,9,FALSE),"")</f>
@@ -5763,7 +5871,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E23">
         <f>IFERROR(VLOOKUP(A23,Modules!$A:$I,9,FALSE),"")</f>
@@ -5795,7 +5903,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E24">
         <f>IFERROR(VLOOKUP(A24,Modules!$A:$I,9,FALSE),"")</f>
@@ -5827,7 +5935,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E25">
         <f>IFERROR(VLOOKUP(A25,Modules!$A:$I,9,FALSE),"")</f>
@@ -5859,7 +5967,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E26">
         <f>IFERROR(VLOOKUP(A26,Modules!$A:$I,9,FALSE),"")</f>
@@ -5891,7 +5999,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E27">
         <f>IFERROR(VLOOKUP(A27,Modules!$A:$I,9,FALSE),"")</f>
@@ -5923,7 +6031,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E28">
         <f>IFERROR(VLOOKUP(A28,Modules!$A:$I,9,FALSE),"")</f>
@@ -5955,7 +6063,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E29">
         <f>IFERROR(VLOOKUP(A29,Modules!$A:$I,9,FALSE),"")</f>
@@ -5987,7 +6095,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E30">
         <f>IFERROR(VLOOKUP(A30,Modules!$A:$I,9,FALSE),"")</f>
@@ -6019,7 +6127,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E31">
         <f>IFERROR(VLOOKUP(A31,Modules!$A:$I,9,FALSE),"")</f>
@@ -6051,7 +6159,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E32">
         <f>IFERROR(VLOOKUP(A32,Modules!$A:$I,9,FALSE),"")</f>
@@ -6083,7 +6191,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E33">
         <f>IFERROR(VLOOKUP(A33,Modules!$A:$I,9,FALSE),"")</f>
@@ -6115,7 +6223,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E34">
         <f>IFERROR(VLOOKUP(A34,Modules!$A:$I,9,FALSE),"")</f>
@@ -6147,7 +6255,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E35">
         <f>IFERROR(VLOOKUP(A35,Modules!$A:$I,9,FALSE),"")</f>
@@ -6179,7 +6287,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E36">
         <f>IFERROR(VLOOKUP(A36,Modules!$A:$I,9,FALSE),"")</f>
@@ -6211,7 +6319,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E37">
         <f>IFERROR(VLOOKUP(A37,Modules!$A:$I,9,FALSE),"")</f>
@@ -6243,7 +6351,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E38">
         <f>IFERROR(VLOOKUP(A38,Modules!$A:$I,9,FALSE),"")</f>
@@ -6275,7 +6383,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E39">
         <f>IFERROR(VLOOKUP(A39,Modules!$A:$I,9,FALSE),"")</f>
@@ -6307,7 +6415,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E40">
         <f>IFERROR(VLOOKUP(A40,Modules!$A:$I,9,FALSE),"")</f>
@@ -6339,7 +6447,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E41">
         <f>IFERROR(VLOOKUP(A41,Modules!$A:$I,9,FALSE),"")</f>
@@ -6371,7 +6479,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E42">
         <f>IFERROR(VLOOKUP(A42,Modules!$A:$I,9,FALSE),"")</f>
@@ -6403,7 +6511,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E43">
         <f>IFERROR(VLOOKUP(A43,Modules!$A:$I,9,FALSE),"")</f>
@@ -6435,7 +6543,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E44">
         <f>IFERROR(VLOOKUP(A44,Modules!$A:$I,9,FALSE),"")</f>
@@ -6467,7 +6575,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E45">
         <f>IFERROR(VLOOKUP(A45,Modules!$A:$I,9,FALSE),"")</f>
@@ -6499,7 +6607,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E46">
         <f>IFERROR(VLOOKUP(A46,Modules!$A:$I,9,FALSE),"")</f>
@@ -6531,7 +6639,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E47">
         <f>IFERROR(VLOOKUP(A47,Modules!$A:$I,9,FALSE),"")</f>
@@ -6563,7 +6671,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E48">
         <f>IFERROR(VLOOKUP(A48,Modules!$A:$I,9,FALSE),"")</f>
@@ -6595,7 +6703,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E49">
         <f>IFERROR(VLOOKUP(A49,Modules!$A:$I,9,FALSE),"")</f>
@@ -6761,7 +6869,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -8204,7 +8312,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
@@ -8276,7 +8384,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
@@ -8564,7 +8672,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
@@ -8636,7 +8744,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
@@ -8708,7 +8816,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
@@ -8780,7 +8888,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
@@ -8852,7 +8960,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
@@ -8924,7 +9032,7 @@
         <v>2</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
@@ -8996,7 +9104,7 @@
         <v>2</v>
       </c>
       <c r="F14" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
@@ -9068,7 +9176,7 @@
         <v>3</v>
       </c>
       <c r="F15" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
@@ -9140,7 +9248,7 @@
         <v>3</v>
       </c>
       <c r="F16" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
@@ -9212,7 +9320,7 @@
         <v>3</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
@@ -9284,7 +9392,7 @@
         <v>3</v>
       </c>
       <c r="F18" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
@@ -9356,7 +9464,7 @@
         <v>4</v>
       </c>
       <c r="F19" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
@@ -9428,7 +9536,7 @@
         <v>4</v>
       </c>
       <c r="F20" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
@@ -9500,7 +9608,7 @@
         <v>4</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
@@ -9572,7 +9680,7 @@
         <v>4</v>
       </c>
       <c r="F22" s="11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
@@ -9644,7 +9752,7 @@
         <v>5</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
@@ -9716,7 +9824,7 @@
         <v>5</v>
       </c>
       <c r="F24" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
@@ -9788,7 +9896,7 @@
         <v>5</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G25" s="11" t="inlineStr">
         <is>
@@ -9860,7 +9968,7 @@
         <v>6</v>
       </c>
       <c r="F26" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
@@ -9932,7 +10040,7 @@
         <v>6</v>
       </c>
       <c r="F27" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G27" s="11" t="inlineStr">
         <is>
@@ -10004,7 +10112,7 @@
         <v>7</v>
       </c>
       <c r="F28" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
@@ -10076,7 +10184,7 @@
         <v>7</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G29" s="11" t="inlineStr">
         <is>
@@ -10148,7 +10256,7 @@
         <v>7</v>
       </c>
       <c r="F30" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
@@ -10220,7 +10328,7 @@
         <v>7</v>
       </c>
       <c r="F31" s="11" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G31" s="11" t="inlineStr">
         <is>
@@ -10292,7 +10400,7 @@
         <v>8</v>
       </c>
       <c r="F32" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
@@ -10364,7 +10472,7 @@
         <v>8</v>
       </c>
       <c r="F33" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G33" s="11" t="inlineStr">
         <is>
@@ -10436,7 +10544,7 @@
         <v>8</v>
       </c>
       <c r="F34" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
@@ -10508,7 +10616,7 @@
         <v>9</v>
       </c>
       <c r="F35" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G35" s="11" t="inlineStr">
         <is>
@@ -10580,7 +10688,7 @@
         <v>9</v>
       </c>
       <c r="F36" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
@@ -10652,7 +10760,7 @@
         <v>9</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G37" s="11" t="inlineStr">
         <is>
@@ -10724,7 +10832,7 @@
         <v>10</v>
       </c>
       <c r="F38" s="11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
@@ -10796,7 +10904,7 @@
         <v>10</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G39" s="11" t="inlineStr">
         <is>
@@ -10868,7 +10976,7 @@
         <v>10</v>
       </c>
       <c r="F40" s="11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
@@ -10940,7 +11048,7 @@
         <v>10</v>
       </c>
       <c r="F41" s="11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G41" s="11" t="inlineStr">
         <is>
@@ -11012,7 +11120,7 @@
         <v>11</v>
       </c>
       <c r="F42" s="11" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
@@ -11084,7 +11192,7 @@
         <v>11</v>
       </c>
       <c r="F43" s="11" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G43" s="11" t="inlineStr">
         <is>
@@ -11156,7 +11264,7 @@
         <v>12</v>
       </c>
       <c r="F44" s="11" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
@@ -11228,7 +11336,7 @@
         <v>12</v>
       </c>
       <c r="F45" s="11" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G45" s="11" t="inlineStr">
         <is>
@@ -11300,7 +11408,7 @@
         <v>12</v>
       </c>
       <c r="F46" s="11" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
@@ -11372,7 +11480,7 @@
         <v>12</v>
       </c>
       <c r="F47" s="11" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G47" s="11" t="inlineStr">
         <is>
@@ -11444,7 +11552,7 @@
         <v>12</v>
       </c>
       <c r="F48" s="11" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
@@ -11516,7 +11624,7 @@
         <v>12</v>
       </c>
       <c r="F49" s="11" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G49" s="11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Rewrite Phase 0 as a from-scratch GenAI learning path (#2)
* Rewrite Phase 0 as a from-scratch GenAI on-ramp

Replace the Staff/Principal-heavy 00-01 chapter with beginner-friendly
GenAI vocabulary, simple diagrams, and a Hello-LLM lab. Reorder Phase 0
to 00-01 → Python/APIs → Math, deferring BankCo/production drills until
after the first model call, and sync roadmap/study/dashboard/tracker.

Co-authored-by: Rahul Chaudhari <rcrahul4@gmail.com>

* Align full curriculum sequencing after GenAI from-scratch on-ramp

Audit and fix navigation/prereq drift so beginners follow
00-01 → Python/APIs → Math → Rules/Agents before Staff+ chapters.
Schedule 00-02/00-03, correct Roadmap Day-1 CTA, Resource Database,
Architecture Index patterns, Career Q maps, broken Related links,
and rebuild the Excel tracker week/project mappings.

Co-authored-by: Rahul Chaudhari <rcrahul4@gmail.com>

---------

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Tracker/GenAI-Masterclass-Tracker.xlsx
+++ b/Tracker/GenAI-Masterclass-Tracker.xlsx
@@ -28,9 +28,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Resources'!$A$1:$O$292</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'SystemDesign'!$A$1:$P$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'LeadershipCareer'!$A$1:$K$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Weekly'!$A$1:$M$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Weekly'!$A$1:$M$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'DailyLog'!$A$1:$N$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Projects'!$A$1:$M$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Projects'!$A$1:$M$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Interviews'!$A$1:$M$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'STAR'!$A$1:$N$9</definedName>
   </definedNames>
@@ -759,7 +759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -850,7 +850,7 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Foundations</t>
+          <t>Foundations — GenAI + craft</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
@@ -860,17 +860,17 @@
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>00-01, 00-02, 00-03</t>
+          <t>00-01, 00-05, 00-06, 00-04</t>
         </is>
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>BankCo decision agent</t>
+          <t>Hello-LLM CLI + FastAPI warmup</t>
         </is>
       </c>
       <c r="F2" s="11" t="inlineStr">
         <is>
-          <t>AI judgment</t>
+          <t>GenAI vocabulary</t>
         </is>
       </c>
       <c r="G2" s="11" t="n">
@@ -883,10 +883,10 @@
         </is>
       </c>
       <c r="J2" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K2" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-05",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-05",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-06",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-06",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-04",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L2" s="13">
@@ -901,27 +901,27 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>LLM Engineering I</t>
+          <t>Foundations — Rules / BankCo</t>
         </is>
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>01 LLM Engineering</t>
+          <t>00 Foundations</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>01-01, 01-02</t>
+          <t>00-02, 00-03</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>Token cost estimator</t>
+          <t>When-not-to-agent memo · BankCo rules</t>
         </is>
       </c>
       <c r="F3" s="11" t="inlineStr">
         <is>
-          <t>Transformer whiteboard</t>
+          <t>Rules vs agent</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
@@ -937,7 +937,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"01-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"01-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-02",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L3" s="13">
@@ -952,7 +952,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>LLM Engineering II</t>
+          <t>LLM Engineering I</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
@@ -962,17 +962,17 @@
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>01-03, 01-04, 01-05</t>
+          <t>01-01, 01-02</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>LiteLLM FastAPI router</t>
+          <t>Token cost estimator</t>
         </is>
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>Inference tradeoffs</t>
+          <t>Transformer whiteboard</t>
         </is>
       </c>
       <c r="G4" s="11" t="n">
@@ -985,10 +985,10 @@
         </is>
       </c>
       <c r="J4" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K4" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"01-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"01-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-04",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"01-05",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-05",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"01-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"01-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-02",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L4" s="13">
@@ -1003,27 +1003,27 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Prompts &amp; Tools</t>
+          <t>LLM Engineering II</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>02 Prompt Engineering</t>
+          <t>01 LLM Engineering</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>02-01, 02-02</t>
+          <t>01-03, 01-04, 01-05</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Structured router agent</t>
+          <t>LiteLLM FastAPI router</t>
         </is>
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>Tool-calling design</t>
+          <t>Inference tradeoffs</t>
         </is>
       </c>
       <c r="G5" s="11" t="n">
@@ -1036,10 +1036,10 @@
         </is>
       </c>
       <c r="J5" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K5" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"02-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"02-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"02-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"02-02",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"01-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"01-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-04",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"01-05",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"01-05",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L5" s="13">
@@ -1054,27 +1054,27 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Agents I</t>
+          <t>Prompts &amp; Tools</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>03 Agentic Fundamentals</t>
+          <t>02 Prompt Engineering</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>03-01, 03-02</t>
+          <t>02-01, 02-02</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Inquiry routing agent</t>
+          <t>Structured router agent</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>Agent loop critique</t>
+          <t>Tool-calling design</t>
         </is>
       </c>
       <c r="G6" s="11" t="n">
@@ -1090,7 +1090,7 @@
         <v>2</v>
       </c>
       <c r="K6" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"03-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"03-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-02",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"02-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"02-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"02-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"02-02",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L6" s="13">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Agents II</t>
+          <t>Agents I</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -1115,17 +1115,17 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>03-03, 03-04</t>
+          <t>03-01, 03-02</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>LangGraph + checkpointing</t>
+          <t>Inquiry routing agent</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>Pattern selection</t>
+          <t>Agent loop critique</t>
         </is>
       </c>
       <c r="G7" s="11" t="n">
@@ -1141,7 +1141,7 @@
         <v>2</v>
       </c>
       <c r="K7" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"03-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"03-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-04",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"03-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"03-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-02",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L7" s="13">
@@ -1156,27 +1156,27 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>RAG I</t>
+          <t>Agents II</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>04 RAG</t>
+          <t>03 Agentic Fundamentals</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>04-01, 04-02</t>
+          <t>03-03, 03-04</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>Ingestion + chunking</t>
+          <t>LangGraph + checkpointing</t>
         </is>
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>Chunking tradeoffs</t>
+          <t>Pattern selection</t>
         </is>
       </c>
       <c r="G8" s="11" t="n">
@@ -1192,7 +1192,7 @@
         <v>2</v>
       </c>
       <c r="K8" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"04-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"04-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-02",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"03-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"03-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"03-04",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L8" s="13">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>RAG II</t>
+          <t>RAG I</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -1217,17 +1217,17 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>04-03, 04-04</t>
+          <t>04-01, 04-02</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Hybrid + rerank + citations</t>
+          <t>Ingestion + chunking</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Hallucination control</t>
+          <t>Chunking tradeoffs</t>
         </is>
       </c>
       <c r="G9" s="11" t="n">
@@ -1243,7 +1243,7 @@
         <v>2</v>
       </c>
       <c r="K9" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"04-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"04-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-04",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"04-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"04-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-02",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L9" s="13">
@@ -1258,31 +1258,31 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>RAG II</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>05 Multi-Agent</t>
+          <t>04 RAG</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>05-01, 05-02, 05-03</t>
+          <t>04-03, 04-04</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Travel planner multi-agent</t>
+          <t>Hybrid + rerank + citations</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>Coordination failures</t>
+          <t>Hallucination control</t>
         </is>
       </c>
       <c r="G10" s="11" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H10" s="11" t="inlineStr"/>
       <c r="I10" s="11" t="inlineStr">
@@ -1291,10 +1291,10 @@
         </is>
       </c>
       <c r="J10" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K10" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"05-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"05-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"05-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"05-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"05-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"05-03",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"04-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"04-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"04-04",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L10" s="13">
@@ -1309,31 +1309,31 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Voice / Multimodal</t>
+          <t>Multi-Agent</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>06 Voice &amp; Multimodal</t>
+          <t>05 Multi-Agent</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>06-01, 06-02</t>
+          <t>05-01, 05-02, 05-03</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>ASR→LLM→TTS bot</t>
+          <t>Travel planner multi-agent</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>Latency budgets</t>
+          <t>Coordination failures</t>
         </is>
       </c>
       <c r="G11" s="11" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H11" s="11" t="inlineStr"/>
       <c r="I11" s="11" t="inlineStr">
@@ -1342,10 +1342,10 @@
         </is>
       </c>
       <c r="J11" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K11" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"06-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"06-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"06-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"06-02",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"05-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"05-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"05-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"05-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"05-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"05-03",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L11" s="13">
@@ -1360,27 +1360,27 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Protocols</t>
+          <t>Voice / Multimodal</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>07 Protocols MCP/A2A</t>
+          <t>06 Voice &amp; Multimodal</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>07-01, 07-02, 07-03</t>
+          <t>06-01, 06-02</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>MCP + A2A negotiation</t>
+          <t>ASR→LLM→TTS bot</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>Protocol design</t>
+          <t>Latency budgets</t>
         </is>
       </c>
       <c r="G12" s="11" t="n">
@@ -1393,10 +1393,10 @@
         </is>
       </c>
       <c r="J12" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K12" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"07-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"07-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"07-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"07-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"07-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"07-03",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"06-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"06-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"06-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"06-02",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L12" s="13">
@@ -1411,27 +1411,27 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Eval / LLMOps</t>
+          <t>Protocols</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>08 Eval &amp; LLMOps</t>
+          <t>07 Protocols MCP/A2A</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>08-01, 08-02, 08-03</t>
+          <t>07-01, 07-02, 07-03, 07-04</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Golden set + ship gate</t>
+          <t>MCP + A2A negotiation</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>Eval strategy</t>
+          <t>Protocol design</t>
         </is>
       </c>
       <c r="G13" s="11" t="n">
@@ -1444,10 +1444,10 @@
         </is>
       </c>
       <c r="J13" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"08-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"08-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"08-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"08-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"08-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"08-03",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"07-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"07-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"07-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"07-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"07-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"07-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"07-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"07-04",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L13" s="13">
@@ -1462,27 +1462,27 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Fine-Tuning</t>
+          <t>Eval / LLMOps</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>09 Fine-Tuning</t>
+          <t>08 Eval &amp; LLMOps</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>09-01, 09-02, 09-03</t>
+          <t>08-01, 08-02, 08-03</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>LoRA compare</t>
+          <t>Golden set + ship gate</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>Prompt vs RAG vs FT</t>
+          <t>Eval strategy</t>
         </is>
       </c>
       <c r="G14" s="11" t="n">
@@ -1498,7 +1498,7 @@
         <v>3</v>
       </c>
       <c r="K14" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"09-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"09-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"09-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"09-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"09-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"09-03",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"08-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"08-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"08-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"08-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"08-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"08-03",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L14" s="13">
@@ -1513,31 +1513,31 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Production Infra</t>
+          <t>Fine-Tuning</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>10 Production Infra</t>
+          <t>09 Fine-Tuning</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>10-01, 10-02, 10-03, 10-04</t>
+          <t>09-01, 09-02, 09-03</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>Dockerized agent API</t>
+          <t>LoRA compare</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>Cost/latency design</t>
+          <t>Prompt vs RAG vs FT</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H15" s="11" t="inlineStr"/>
       <c r="I15" s="11" t="inlineStr">
@@ -1546,10 +1546,10 @@
         </is>
       </c>
       <c r="J15" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K15" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"10-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"10-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"10-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"10-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-04",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"09-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"09-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"09-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"09-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"09-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"09-03",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L15" s="13">
@@ -1564,27 +1564,27 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Security + Advanced</t>
+          <t>Production Infra</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>11 Security &amp; Safety</t>
+          <t>10 Production Infra</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>11-01, 11-02, 12-01, 12-02</t>
+          <t>10-01, 10-02, 10-03, 10-04</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Red-team + Text2SQL</t>
+          <t>Dockerized agent API</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Safety review</t>
+          <t>Cost/latency design</t>
         </is>
       </c>
       <c r="G16" s="11" t="n">
@@ -1600,7 +1600,7 @@
         <v>4</v>
       </c>
       <c r="K16" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"11-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"11-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"11-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"11-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-02",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"10-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"10-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"10-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"10-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"10-04",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L16" s="13">
@@ -1615,27 +1615,27 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Advanced + Capstone</t>
+          <t>Security + Advanced</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>12 Advanced Topics</t>
+          <t>11 Security &amp; Safety</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>12-03, 12-04</t>
+          <t>11-01, 11-02, 12-01, 12-02</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>Capstone vertical slice</t>
+          <t>Red-team + Text2SQL</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>Full design interview</t>
+          <t>Safety review</t>
         </is>
       </c>
       <c r="G17" s="11" t="n">
@@ -1648,10 +1648,10 @@
         </is>
       </c>
       <c r="J17" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K17" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"12-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-04",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"11-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"11-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"11-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"11-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-02",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L17" s="13">
@@ -1666,31 +1666,31 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Capstone + Mocks</t>
+          <t>Advanced + Capstone</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Capstone</t>
+          <t>12 Advanced Topics</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>CAPSTONE</t>
+          <t>12-03, 12-04, 12-05, 12-06</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Capstone v1 + 4 mocks</t>
+          <t>Capstone vertical slice</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>Panel simulation</t>
+          <t>Full design interview</t>
         </is>
       </c>
       <c r="G18" s="11" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H18" s="11" t="inlineStr"/>
       <c r="I18" s="11" t="inlineStr">
@@ -1699,10 +1699,10 @@
         </is>
       </c>
       <c r="J18" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K18" s="11">
-        <f>COUNTIFS(Projects!D:D,"Capstone",Projects!F:F,"Done")+COUNTIFS(Projects!D:D,"Capstone",Projects!F:F,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"12-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-04",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-05",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-05",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"12-06",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"12-06",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L18" s="13">
@@ -1711,10 +1711,61 @@
       </c>
       <c r="M18" s="11" t="n"/>
     </row>
+    <row r="19">
+      <c r="A19" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Capstone + Mocks</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Capstone</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>CAPSTONE</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Capstone v1 + 4 mocks</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Panel simulation</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="H19" s="11" t="inlineStr"/>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="11">
+        <f>COUNTIFS(Projects!D:D,"Capstone",Projects!F:F,"Done")+COUNTIFS(Projects!D:D,"Capstone",Projects!F:F,"Interview-ready")</f>
+        <v/>
+      </c>
+      <c r="L19" s="13">
+        <f>IF(J19=0,"",K19/J19)</f>
+        <v/>
+      </c>
+      <c r="M19" s="11" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M18"/>
+  <autoFilter ref="A1:M19"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Done,Interview-ready"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3289,7 +3340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3382,7 +3433,7 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>BankCo Decision Support</t>
+          <t>Hello-LLM Explain-It Bot</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
@@ -3405,7 +3456,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>00-01, 00-03</t>
+          <t>00-01</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr"/>
@@ -3434,17 +3485,17 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>P01b</t>
         </is>
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>Token Cost Estimator</t>
+          <t>BankCo Decision Support</t>
         </is>
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>LLM Projects</t>
+          <t>Foundations Projects</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
@@ -3462,7 +3513,7 @@
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
-          <t>01-02</t>
+          <t>00-02, 00-03</t>
         </is>
       </c>
       <c r="H3" s="11" t="inlineStr"/>
@@ -3491,12 +3542,12 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>P03</t>
+          <t>P02</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>LiteLLM Gateway</t>
+          <t>Token Cost Estimator</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
@@ -3519,7 +3570,7 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>01-04, 01-05</t>
+          <t>01-02</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr"/>
@@ -3548,22 +3599,22 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>P04</t>
+          <t>P03</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Structured Router Agent</t>
+          <t>LiteLLM Gateway</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Agent Projects</t>
+          <t>LLM Projects</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Mini</t>
         </is>
       </c>
       <c r="E5" s="11" t="n">
@@ -3576,7 +3627,7 @@
       </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
-          <t>02-02, 03-03</t>
+          <t>01-04, 01-05</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr"/>
@@ -3605,12 +3656,12 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P04</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Inquiry Routing Agent</t>
+          <t>Structured Router Agent</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -3633,7 +3684,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>03-01, 03-02</t>
+          <t>02-02, 03-03</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr"/>
@@ -3662,12 +3713,12 @@
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>P06</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>LangGraph Production Agent</t>
+          <t>Inquiry Routing Agent</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -3690,7 +3741,7 @@
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
-          <t>03-04</t>
+          <t>03-01, 03-02</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr"/>
@@ -3719,26 +3770,26 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>P06</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>NovaCart RAG Assistant</t>
+          <t>LangGraph Production Agent</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>RAG Projects</t>
+          <t>Agent Projects</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="E8" s="11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
@@ -3747,7 +3798,7 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>04-01, 04-02, 04-03</t>
+          <t>03-04</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr"/>
@@ -3776,17 +3827,17 @@
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Multi-Agent Travel Planner</t>
+          <t>NovaCart RAG Assistant</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Multi-Agent Projects</t>
+          <t>RAG Projects</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
@@ -3804,7 +3855,7 @@
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>05-01, 05-02</t>
+          <t>04-01, 04-02, 04-03</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr"/>
@@ -3833,22 +3884,22 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Voice Bot</t>
+          <t>Multi-Agent Travel Planner</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Multimodal Projects</t>
+          <t>Multi-Agent Projects</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
@@ -3861,7 +3912,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>06-01</t>
+          <t>05-01, 05-02</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr"/>
@@ -3890,22 +3941,22 @@
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>MCP + Negotiation Sim</t>
+          <t>Voice Bot</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Protocol Projects</t>
+          <t>Multimodal Projects</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
@@ -3918,7 +3969,7 @@
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>07-01, 07-02, 07-03</t>
+          <t>06-01</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr"/>
@@ -3947,17 +3998,17 @@
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Eval Harness + Ship Gate</t>
+          <t>MCP + Negotiation Sim</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>LLMOps Projects</t>
+          <t>Protocol Projects</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -3975,7 +4026,7 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>08-01, 08-03</t>
+          <t>07-01, 07-02, 07-03</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr"/>
@@ -4004,22 +4055,22 @@
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>LoRA Integration</t>
+          <t>Eval Harness + Ship Gate</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Fine-Tune Projects</t>
+          <t>LLMOps Projects</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="E13" s="11" t="n">
@@ -4032,7 +4083,7 @@
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>09-01, 09-02, 09-03</t>
+          <t>08-01, 08-03</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr"/>
@@ -4061,22 +4112,22 @@
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>P13</t>
+          <t>P12</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Deployed Agent API</t>
+          <t>LoRA Integration</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Infra Projects</t>
+          <t>Fine-Tune Projects</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="E14" s="11" t="n">
@@ -4089,7 +4140,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>10-01, 10-02, 10-04</t>
+          <t>09-01, 09-02, 09-03</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr"/>
@@ -4118,26 +4169,26 @@
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>P13</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Capstone Multi-Agent System</t>
+          <t>Deployed Agent API</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Capstone</t>
+          <t>Infra Projects</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Capstone</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
@@ -4146,7 +4197,7 @@
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>05-01, 04-01, 08-01, 11-01</t>
+          <t>10-01, 10-02, 10-04</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr"/>
@@ -4172,9 +4223,66 @@
       </c>
       <c r="M15" s="11" t="inlineStr"/>
     </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Capstone Multi-Agent System</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Capstone</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Capstone</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>05-01, 04-01, 08-01, 11-01</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr"/>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K16" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L16" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M16" s="11" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M15"/>
-  <conditionalFormatting sqref="F2:F15">
+  <autoFilter ref="A1:M16"/>
+  <conditionalFormatting sqref="F2:F16">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F2="Done"</formula>
     </cfRule>
@@ -4183,22 +4291,22 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
-    <dataValidation sqref="F2:F15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Done,Interview-ready"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Mini,Intermediate,Production,Capstone"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4699,7 +4807,7 @@
       <c r="G2" s="11" t="inlineStr"/>
       <c r="H2" s="11" t="inlineStr">
         <is>
-          <t>00-01, 08-03</t>
+          <t>12-06, 08-03</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr"/>
@@ -4963,7 +5071,7 @@
       <c r="G8" s="11" t="inlineStr"/>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>00-01</t>
+          <t>12-06</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr"/>
@@ -5082,7 +5190,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>00-01 — AI Engineering Mindset for Principal, Staff &amp; Engineering Managers</t>
+          <t>00-01 — GenAI From Scratch: Core Ideas</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -5123,7 +5231,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <f>IFERROR(VLOOKUP(A3,Modules!$A:$I,9,FALSE),"")</f>
@@ -5155,7 +5263,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <f>IFERROR(VLOOKUP(A4,Modules!$A:$I,9,FALSE),"")</f>
@@ -5283,7 +5391,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8">
         <f>IFERROR(VLOOKUP(A8,Modules!$A:$I,9,FALSE),"")</f>
@@ -5315,7 +5423,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9">
         <f>IFERROR(VLOOKUP(A9,Modules!$A:$I,9,FALSE),"")</f>
@@ -5347,7 +5455,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10">
         <f>IFERROR(VLOOKUP(A10,Modules!$A:$I,9,FALSE),"")</f>
@@ -5379,7 +5487,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11">
         <f>IFERROR(VLOOKUP(A11,Modules!$A:$I,9,FALSE),"")</f>
@@ -5411,7 +5519,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12">
         <f>IFERROR(VLOOKUP(A12,Modules!$A:$I,9,FALSE),"")</f>
@@ -5443,7 +5551,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E13">
         <f>IFERROR(VLOOKUP(A13,Modules!$A:$I,9,FALSE),"")</f>
@@ -5475,7 +5583,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E14">
         <f>IFERROR(VLOOKUP(A14,Modules!$A:$I,9,FALSE),"")</f>
@@ -5507,7 +5615,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E15">
         <f>IFERROR(VLOOKUP(A15,Modules!$A:$I,9,FALSE),"")</f>
@@ -5539,7 +5647,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E16">
         <f>IFERROR(VLOOKUP(A16,Modules!$A:$I,9,FALSE),"")</f>
@@ -5571,7 +5679,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E17">
         <f>IFERROR(VLOOKUP(A17,Modules!$A:$I,9,FALSE),"")</f>
@@ -5603,7 +5711,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E18">
         <f>IFERROR(VLOOKUP(A18,Modules!$A:$I,9,FALSE),"")</f>
@@ -5635,7 +5743,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E19">
         <f>IFERROR(VLOOKUP(A19,Modules!$A:$I,9,FALSE),"")</f>
@@ -5667,7 +5775,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E20">
         <f>IFERROR(VLOOKUP(A20,Modules!$A:$I,9,FALSE),"")</f>
@@ -5699,7 +5807,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E21">
         <f>IFERROR(VLOOKUP(A21,Modules!$A:$I,9,FALSE),"")</f>
@@ -5731,7 +5839,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E22">
         <f>IFERROR(VLOOKUP(A22,Modules!$A:$I,9,FALSE),"")</f>
@@ -5763,7 +5871,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E23">
         <f>IFERROR(VLOOKUP(A23,Modules!$A:$I,9,FALSE),"")</f>
@@ -5795,7 +5903,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E24">
         <f>IFERROR(VLOOKUP(A24,Modules!$A:$I,9,FALSE),"")</f>
@@ -5827,7 +5935,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E25">
         <f>IFERROR(VLOOKUP(A25,Modules!$A:$I,9,FALSE),"")</f>
@@ -5859,7 +5967,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E26">
         <f>IFERROR(VLOOKUP(A26,Modules!$A:$I,9,FALSE),"")</f>
@@ -5891,7 +5999,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E27">
         <f>IFERROR(VLOOKUP(A27,Modules!$A:$I,9,FALSE),"")</f>
@@ -5923,7 +6031,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E28">
         <f>IFERROR(VLOOKUP(A28,Modules!$A:$I,9,FALSE),"")</f>
@@ -5955,7 +6063,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E29">
         <f>IFERROR(VLOOKUP(A29,Modules!$A:$I,9,FALSE),"")</f>
@@ -5987,7 +6095,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E30">
         <f>IFERROR(VLOOKUP(A30,Modules!$A:$I,9,FALSE),"")</f>
@@ -6019,7 +6127,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E31">
         <f>IFERROR(VLOOKUP(A31,Modules!$A:$I,9,FALSE),"")</f>
@@ -6051,7 +6159,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E32">
         <f>IFERROR(VLOOKUP(A32,Modules!$A:$I,9,FALSE),"")</f>
@@ -6083,7 +6191,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E33">
         <f>IFERROR(VLOOKUP(A33,Modules!$A:$I,9,FALSE),"")</f>
@@ -6115,7 +6223,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E34">
         <f>IFERROR(VLOOKUP(A34,Modules!$A:$I,9,FALSE),"")</f>
@@ -6147,7 +6255,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E35">
         <f>IFERROR(VLOOKUP(A35,Modules!$A:$I,9,FALSE),"")</f>
@@ -6179,7 +6287,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E36">
         <f>IFERROR(VLOOKUP(A36,Modules!$A:$I,9,FALSE),"")</f>
@@ -6211,7 +6319,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E37">
         <f>IFERROR(VLOOKUP(A37,Modules!$A:$I,9,FALSE),"")</f>
@@ -6243,7 +6351,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E38">
         <f>IFERROR(VLOOKUP(A38,Modules!$A:$I,9,FALSE),"")</f>
@@ -6275,7 +6383,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E39">
         <f>IFERROR(VLOOKUP(A39,Modules!$A:$I,9,FALSE),"")</f>
@@ -6307,7 +6415,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E40">
         <f>IFERROR(VLOOKUP(A40,Modules!$A:$I,9,FALSE),"")</f>
@@ -6339,7 +6447,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E41">
         <f>IFERROR(VLOOKUP(A41,Modules!$A:$I,9,FALSE),"")</f>
@@ -6371,7 +6479,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E42">
         <f>IFERROR(VLOOKUP(A42,Modules!$A:$I,9,FALSE),"")</f>
@@ -6403,7 +6511,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E43">
         <f>IFERROR(VLOOKUP(A43,Modules!$A:$I,9,FALSE),"")</f>
@@ -6435,7 +6543,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E44">
         <f>IFERROR(VLOOKUP(A44,Modules!$A:$I,9,FALSE),"")</f>
@@ -6467,7 +6575,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E45">
         <f>IFERROR(VLOOKUP(A45,Modules!$A:$I,9,FALSE),"")</f>
@@ -6499,7 +6607,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E46">
         <f>IFERROR(VLOOKUP(A46,Modules!$A:$I,9,FALSE),"")</f>
@@ -6531,7 +6639,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E47">
         <f>IFERROR(VLOOKUP(A47,Modules!$A:$I,9,FALSE),"")</f>
@@ -6563,7 +6671,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E48">
         <f>IFERROR(VLOOKUP(A48,Modules!$A:$I,9,FALSE),"")</f>
@@ -6595,7 +6703,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E49">
         <f>IFERROR(VLOOKUP(A49,Modules!$A:$I,9,FALSE),"")</f>
@@ -6761,7 +6869,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -8115,7 +8223,7 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>00-01 — AI Engineering Mindset for Principal, Staff &amp; Engineering Managers</t>
+          <t>00-01 — GenAI From Scratch: Core Ideas</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
@@ -8140,7 +8248,7 @@
         </is>
       </c>
       <c r="H2" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
@@ -8204,7 +8312,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
@@ -8276,7 +8384,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
@@ -8564,7 +8672,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
@@ -8636,7 +8744,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
@@ -8708,7 +8816,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
@@ -8780,7 +8888,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
@@ -8852,7 +8960,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
@@ -8924,7 +9032,7 @@
         <v>2</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
@@ -8996,7 +9104,7 @@
         <v>2</v>
       </c>
       <c r="F14" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
@@ -9068,7 +9176,7 @@
         <v>3</v>
       </c>
       <c r="F15" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
@@ -9140,7 +9248,7 @@
         <v>3</v>
       </c>
       <c r="F16" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
@@ -9212,7 +9320,7 @@
         <v>3</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
@@ -9284,7 +9392,7 @@
         <v>3</v>
       </c>
       <c r="F18" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
@@ -9356,7 +9464,7 @@
         <v>4</v>
       </c>
       <c r="F19" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
@@ -9428,7 +9536,7 @@
         <v>4</v>
       </c>
       <c r="F20" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
@@ -9500,7 +9608,7 @@
         <v>4</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
@@ -9572,7 +9680,7 @@
         <v>4</v>
       </c>
       <c r="F22" s="11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
@@ -9644,7 +9752,7 @@
         <v>5</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
@@ -9716,7 +9824,7 @@
         <v>5</v>
       </c>
       <c r="F24" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
@@ -9788,7 +9896,7 @@
         <v>5</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G25" s="11" t="inlineStr">
         <is>
@@ -9860,7 +9968,7 @@
         <v>6</v>
       </c>
       <c r="F26" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
@@ -9932,7 +10040,7 @@
         <v>6</v>
       </c>
       <c r="F27" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G27" s="11" t="inlineStr">
         <is>
@@ -10004,7 +10112,7 @@
         <v>7</v>
       </c>
       <c r="F28" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
@@ -10076,7 +10184,7 @@
         <v>7</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G29" s="11" t="inlineStr">
         <is>
@@ -10148,7 +10256,7 @@
         <v>7</v>
       </c>
       <c r="F30" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
@@ -10220,7 +10328,7 @@
         <v>7</v>
       </c>
       <c r="F31" s="11" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G31" s="11" t="inlineStr">
         <is>
@@ -10292,7 +10400,7 @@
         <v>8</v>
       </c>
       <c r="F32" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
@@ -10364,7 +10472,7 @@
         <v>8</v>
       </c>
       <c r="F33" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G33" s="11" t="inlineStr">
         <is>
@@ -10436,7 +10544,7 @@
         <v>8</v>
       </c>
       <c r="F34" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
@@ -10508,7 +10616,7 @@
         <v>9</v>
       </c>
       <c r="F35" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G35" s="11" t="inlineStr">
         <is>
@@ -10580,7 +10688,7 @@
         <v>9</v>
       </c>
       <c r="F36" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
@@ -10652,7 +10760,7 @@
         <v>9</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G37" s="11" t="inlineStr">
         <is>
@@ -10724,7 +10832,7 @@
         <v>10</v>
       </c>
       <c r="F38" s="11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
@@ -10796,7 +10904,7 @@
         <v>10</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G39" s="11" t="inlineStr">
         <is>
@@ -10868,7 +10976,7 @@
         <v>10</v>
       </c>
       <c r="F40" s="11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
@@ -10940,7 +11048,7 @@
         <v>10</v>
       </c>
       <c r="F41" s="11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G41" s="11" t="inlineStr">
         <is>
@@ -11012,7 +11120,7 @@
         <v>11</v>
       </c>
       <c r="F42" s="11" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
@@ -11084,7 +11192,7 @@
         <v>11</v>
       </c>
       <c r="F43" s="11" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G43" s="11" t="inlineStr">
         <is>
@@ -11156,7 +11264,7 @@
         <v>12</v>
       </c>
       <c r="F44" s="11" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
@@ -11228,7 +11336,7 @@
         <v>12</v>
       </c>
       <c r="F45" s="11" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G45" s="11" t="inlineStr">
         <is>
@@ -11300,7 +11408,7 @@
         <v>12</v>
       </c>
       <c r="F46" s="11" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
@@ -11372,7 +11480,7 @@
         <v>12</v>
       </c>
       <c r="F47" s="11" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G47" s="11" t="inlineStr">
         <is>
@@ -11444,7 +11552,7 @@
         <v>12</v>
       </c>
       <c r="F48" s="11" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
@@ -11516,7 +11624,7 @@
         <v>12</v>
       </c>
       <c r="F49" s="11" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G49" s="11" t="inlineStr">
         <is>
@@ -11721,12 +11829,12 @@
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>LangGraph Overview</t>
+          <t>OpenAI — Text generation / chat concepts</t>
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr">
         <is>
-          <t>https://langchain-ai.github.io/langgraph/concepts/high_level/</t>
+          <t>https://platform.openai.com/docs/guides/text</t>
         </is>
       </c>
       <c r="G2" s="12">
@@ -11744,17 +11852,17 @@
       </c>
       <c r="J2" s="11" t="inlineStr">
         <is>
-          <t>20 min</t>
+          <t>20–30 min</t>
         </is>
       </c>
       <c r="K2" s="11" t="inlineStr">
         <is>
-          <t>See production agent runtime concerns (persistence, HITL)</t>
+          <t>Solidify messages, models, tokens</t>
         </is>
       </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>Core benefits; ecosystem; persistence</t>
+          <t>Messages; models; token basics</t>
         </is>
       </c>
       <c r="M2" s="11" t="inlineStr">
@@ -11790,12 +11898,12 @@
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>MCP Intro</t>
+          <t>Anthropic — Claude overview</t>
         </is>
       </c>
       <c r="F3" s="12" t="inlineStr">
         <is>
-          <t>https://modelcontextprotocol.io/docs/getting-started/intro</t>
+          <t>https://docs.anthropic.com/en/docs/welcome</t>
         </is>
       </c>
       <c r="G3" s="12">
@@ -11813,17 +11921,17 @@
       </c>
       <c r="J3" s="11" t="inlineStr">
         <is>
-          <t>15 min</t>
+          <t>20 min</t>
         </is>
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>Standard tool connectivity mindset</t>
+          <t>Second provider vocabulary</t>
         </is>
       </c>
       <c r="L3" s="11" t="inlineStr">
         <is>
-          <t>What MCP enables; why it matters</t>
+          <t>Messages API mental model</t>
         </is>
       </c>
       <c r="M3" s="11" t="inlineStr">
@@ -11859,12 +11967,12 @@
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>OpenAI Prompt Engineering Guide</t>
+          <t>Google — Gemini API quickstart</t>
         </is>
       </c>
       <c r="F4" s="12" t="inlineStr">
         <is>
-          <t>https://developers.openai.com/api/docs/guides/prompt-engineering</t>
+          <t>https://ai.google.dev/gemini-api/docs/quickstart</t>
         </is>
       </c>
       <c r="G4" s="12">
@@ -11882,17 +11990,17 @@
       </c>
       <c r="J4" s="11" t="inlineStr">
         <is>
-          <t>45 min</t>
+          <t>20 min</t>
         </is>
       </c>
       <c r="K4" s="11" t="inlineStr">
         <is>
-          <t>Prompt as contract, not poetry</t>
+          <t>Multi-provider habit early</t>
         </is>
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Tactics; message roles; iteration</t>
+          <t>First request</t>
         </is>
       </c>
       <c r="M4" s="11" t="inlineStr">
@@ -11928,12 +12036,12 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Anthropic / Claude Docs Overview</t>
+          <t>DeepSeek API docs</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>https://platform.claude.com/docs/en/docs/build-with-claude/overview</t>
+          <t>https://api-docs.deepseek.com/</t>
         </is>
       </c>
       <c r="G5" s="12">
@@ -11951,17 +12059,17 @@
       </c>
       <c r="J5" s="11" t="inlineStr">
         <is>
-          <t>30 min</t>
+          <t>15 min</t>
         </is>
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>Alternate provider constraints</t>
+          <t>Cost-efficient OpenAI-compatible option</t>
         </is>
       </c>
       <c r="L5" s="11" t="inlineStr">
         <is>
-          <t>Build with Claude overview</t>
+          <t>First chat call</t>
         </is>
       </c>
       <c r="M5" s="11" t="inlineStr">
@@ -11997,12 +12105,12 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Attention Is All You Need</t>
+          <t>OpenAI Prompt Engineering Guide</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/1706.03762</t>
+          <t>https://developers.openai.com/api/docs/guides/prompt-engineering</t>
         </is>
       </c>
       <c r="G6" s="12">
@@ -12015,22 +12123,22 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Intro</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
         <is>
-          <t>60–90 min</t>
+          <t>45 min</t>
         </is>
       </c>
       <c r="K6" s="11" t="inlineStr">
         <is>
-          <t>Shared vocabulary for later chapters</t>
+          <t>Prompts as clear instructions</t>
         </is>
       </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>Architecture diagram; attention</t>
+          <t>Tactics; iteration</t>
         </is>
       </c>
       <c r="M6" s="11" t="inlineStr">
@@ -12066,12 +12174,12 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>ReAct: Synergizing Reasoning and Acting</t>
+          <t>Chip Huyen — *AI Engineering* (book)</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2210.03629</t>
+          <t>https://www.oreilly.com/library/view/ai-engineering/9781098166298/</t>
         </is>
       </c>
       <c r="G7" s="12">
@@ -12089,17 +12197,17 @@
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>45 min</t>
+          <t>ongoing</t>
         </is>
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>Grounds the agent loop chapter</t>
+          <t>Bridge from ideas to production later</t>
         </is>
       </c>
       <c r="L7" s="11" t="inlineStr">
         <is>
-          <t>Think-Act-Observe examples</t>
+          <t>Early chapters on AI eng vs ML eng</t>
         </is>
       </c>
       <c r="M7" s="11" t="inlineStr">
@@ -12135,12 +12243,12 @@
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>OWASP Top 10 for LLM Applications</t>
+          <t>Karpathy — Intro to LLMs (talk)</t>
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>https://owasp.org/www-project-top-10-for-large-language-model-applications/</t>
+          <t>https://www.youtube.com/watch?v=zjkBMFhNj_g</t>
         </is>
       </c>
       <c r="G8" s="12">
@@ -12153,7 +12261,7 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Intro</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
@@ -12163,12 +12271,12 @@
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>Safety mindset early</t>
+          <t>Intuition without heavy math</t>
         </is>
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>LLM01 Prompt Injection; data leakage</t>
+          <t>Whole talk once</t>
         </is>
       </c>
       <c r="M8" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Renumber Module 00 so IDs match Track D study order
Foundation chapters are now 00-01 GenAI → 00-02 Python → 00-03 APIs →
00-04 Rules→Agents → 00-05 Math → 00-06 BankCo. Update nav docs, links,
diagrams, and tracker so numbering is the learning path—not a catalog
mismatch.

Co-authored-by: Rahul Chaudhari <rcrahul4@gmail.com>
</commit_message>
<xml_diff>
--- a/Tracker/GenAI-Masterclass-Tracker.xlsx
+++ b/Tracker/GenAI-Masterclass-Tracker.xlsx
@@ -27,7 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Modules'!$A$1:$R$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Resources'!$A$1:$O$292</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'SystemDesign'!$A$1:$P$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'LeadershipCareer'!$A$1:$K$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'LeadershipCareer'!$A$1:$K$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Weekly'!$A$1:$M$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'DailyLog'!$A$1:$N$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Projects'!$A$1:$M$16</definedName>
@@ -860,7 +860,7 @@
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>00-01, 00-05, 00-06, 00-04</t>
+          <t>00-01, 00-02, 00-03, 00-05</t>
         </is>
       </c>
       <c r="E2" s="11" t="inlineStr">
@@ -886,7 +886,7 @@
         <v>4</v>
       </c>
       <c r="K2" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-05",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-05",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-06",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-06",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-04",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-05",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-05",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L2" s="13">
@@ -911,7 +911,7 @@
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>00-02, 00-03</t>
+          <t>00-04, 00-06</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
@@ -937,7 +937,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"00-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-04",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-06",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-06",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L3" s="13">
@@ -3513,7 +3513,7 @@
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
-          <t>00-02, 00-03</t>
+          <t>00-04, 00-06</t>
         </is>
       </c>
       <c r="H3" s="11" t="inlineStr"/>
@@ -5222,7 +5222,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>00-02 — From Rules to Agents: The Evolution of Intelligent Systems</t>
+          <t>00-02 — Python for AI Engineering</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5231,7 +5231,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3">
         <f>IFERROR(VLOOKUP(A3,Modules!$A:$I,9,FALSE),"")</f>
@@ -5254,7 +5254,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>00-03 — BankCo Warm-Up: Decision-Support Retention Assistant</t>
+          <t>00-03 — APIs for AI Engineering</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -5263,7 +5263,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4">
         <f>IFERROR(VLOOKUP(A4,Modules!$A:$I,9,FALSE),"")</f>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>00-04 — Mathematics for AI Engineering</t>
+          <t>00-04 — From Rules to Agents: The Evolution of Intelligent Systems</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -5295,7 +5295,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <f>IFERROR(VLOOKUP(A5,Modules!$A:$I,9,FALSE),"")</f>
@@ -5318,7 +5318,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>00-05 — Python for AI Engineering</t>
+          <t>00-05 — Mathematics for AI Engineering</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -5350,7 +5350,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>00-06 — APIs for AI Engineering</t>
+          <t>00-06 — BankCo Warm-Up: Decision-Support Retention Assistant</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -5359,7 +5359,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7">
         <f>IFERROR(VLOOKUP(A7,Modules!$A:$I,9,FALSE),"")</f>
@@ -8274,7 +8274,7 @@
       <c r="N2" s="11" t="inlineStr"/>
       <c r="O2" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-01-AI-Engineering-Mindset.md</t>
+          <t>Modules/00-Foundations/00-01-GenAI-From-Scratch.md</t>
         </is>
       </c>
       <c r="P2" s="12">
@@ -8295,7 +8295,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>00-02 — From Rules to Agents: The Evolution of Intelligent Systems</t>
+          <t>00-02 — Python for AI Engineering</t>
         </is>
       </c>
       <c r="C3" s="11" t="inlineStr">
@@ -8312,7 +8312,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
@@ -8346,7 +8346,7 @@
       <c r="N3" s="11" t="inlineStr"/>
       <c r="O3" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-02-From-Rules-to-Agents.md</t>
+          <t>Modules/00-Foundations/00-02-Python-for-AI-Engineering.md</t>
         </is>
       </c>
       <c r="P3" s="12">
@@ -8367,7 +8367,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>00-03 — BankCo Warm-Up: Decision-Support Retention Assistant</t>
+          <t>00-03 — APIs for AI Engineering</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
@@ -8384,7 +8384,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
@@ -8392,7 +8392,7 @@
         </is>
       </c>
       <c r="H4" s="11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
@@ -8418,7 +8418,7 @@
       <c r="N4" s="11" t="inlineStr"/>
       <c r="O4" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-03-BankCo-Decision-Support-Warmup.md</t>
+          <t>Modules/00-Foundations/00-03-APIs-for-AI-Engineering.md</t>
         </is>
       </c>
       <c r="P4" s="12">
@@ -8439,7 +8439,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>00-04 — Mathematics for AI Engineering</t>
+          <t>00-04 — From Rules to Agents: The Evolution of Intelligent Systems</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
@@ -8456,7 +8456,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
@@ -8464,7 +8464,7 @@
         </is>
       </c>
       <c r="H5" s="11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
@@ -8490,7 +8490,7 @@
       <c r="N5" s="11" t="inlineStr"/>
       <c r="O5" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-04-Mathematics-for-AI-Engineering.md</t>
+          <t>Modules/00-Foundations/00-04-From-Rules-to-Agents.md</t>
         </is>
       </c>
       <c r="P5" s="12">
@@ -8511,7 +8511,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>00-05 — Python for AI Engineering</t>
+          <t>00-05 — Mathematics for AI Engineering</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -8536,7 +8536,7 @@
         </is>
       </c>
       <c r="H6" s="11" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
@@ -8562,7 +8562,7 @@
       <c r="N6" s="11" t="inlineStr"/>
       <c r="O6" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-05-Python-for-AI-Engineering.md</t>
+          <t>Modules/00-Foundations/00-05-Mathematics-for-AI-Engineering.md</t>
         </is>
       </c>
       <c r="P6" s="12">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>00-06 — APIs for AI Engineering</t>
+          <t>00-06 — BankCo Warm-Up: Decision-Support Retention Assistant</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -8600,7 +8600,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
@@ -8608,7 +8608,7 @@
         </is>
       </c>
       <c r="H7" s="11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
@@ -8634,7 +8634,7 @@
       <c r="N7" s="11" t="inlineStr"/>
       <c r="O7" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-06-APIs-for-AI-Engineering.md</t>
+          <t>Modules/00-Foundations/00-06-BankCo-Decision-Support-Warmup.md</t>
         </is>
       </c>
       <c r="P7" s="12">
@@ -11867,7 +11867,7 @@
       </c>
       <c r="M2" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-01-AI-Engineering-Mindset.md</t>
+          <t>Modules/00-Foundations/00-01-GenAI-From-Scratch.md</t>
         </is>
       </c>
       <c r="N2" s="11" t="inlineStr">
@@ -11936,7 +11936,7 @@
       </c>
       <c r="M3" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-01-AI-Engineering-Mindset.md</t>
+          <t>Modules/00-Foundations/00-01-GenAI-From-Scratch.md</t>
         </is>
       </c>
       <c r="N3" s="11" t="inlineStr">
@@ -12005,7 +12005,7 @@
       </c>
       <c r="M4" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-01-AI-Engineering-Mindset.md</t>
+          <t>Modules/00-Foundations/00-01-GenAI-From-Scratch.md</t>
         </is>
       </c>
       <c r="N4" s="11" t="inlineStr">
@@ -12074,7 +12074,7 @@
       </c>
       <c r="M5" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-01-AI-Engineering-Mindset.md</t>
+          <t>Modules/00-Foundations/00-01-GenAI-From-Scratch.md</t>
         </is>
       </c>
       <c r="N5" s="11" t="inlineStr">
@@ -12143,7 +12143,7 @@
       </c>
       <c r="M6" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-01-AI-Engineering-Mindset.md</t>
+          <t>Modules/00-Foundations/00-01-GenAI-From-Scratch.md</t>
         </is>
       </c>
       <c r="N6" s="11" t="inlineStr">
@@ -12212,7 +12212,7 @@
       </c>
       <c r="M7" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-01-AI-Engineering-Mindset.md</t>
+          <t>Modules/00-Foundations/00-01-GenAI-From-Scratch.md</t>
         </is>
       </c>
       <c r="N7" s="11" t="inlineStr">
@@ -12281,7 +12281,7 @@
       </c>
       <c r="M8" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-01-AI-Engineering-Mindset.md</t>
+          <t>Modules/00-Foundations/00-01-GenAI-From-Scratch.md</t>
         </is>
       </c>
       <c r="N8" s="11" t="inlineStr">
@@ -12299,7 +12299,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>00-02</t>
+          <t>00-04</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -12350,7 +12350,7 @@
       </c>
       <c r="M9" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-02-From-Rules-to-Agents.md</t>
+          <t>Modules/00-Foundations/00-04-From-Rules-to-Agents.md</t>
         </is>
       </c>
       <c r="N9" s="11" t="inlineStr">
@@ -12368,7 +12368,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>00-02</t>
+          <t>00-04</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -12419,7 +12419,7 @@
       </c>
       <c r="M10" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-02-From-Rules-to-Agents.md</t>
+          <t>Modules/00-Foundations/00-04-From-Rules-to-Agents.md</t>
         </is>
       </c>
       <c r="N10" s="11" t="inlineStr">
@@ -12437,7 +12437,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>00-02</t>
+          <t>00-04</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
@@ -12488,7 +12488,7 @@
       </c>
       <c r="M11" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-02-From-Rules-to-Agents.md</t>
+          <t>Modules/00-Foundations/00-04-From-Rules-to-Agents.md</t>
         </is>
       </c>
       <c r="N11" s="11" t="inlineStr">
@@ -12506,7 +12506,7 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>00-02</t>
+          <t>00-04</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -12557,7 +12557,7 @@
       </c>
       <c r="M12" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-02-From-Rules-to-Agents.md</t>
+          <t>Modules/00-Foundations/00-04-From-Rules-to-Agents.md</t>
         </is>
       </c>
       <c r="N12" s="11" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>00-02</t>
+          <t>00-04</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
@@ -12626,7 +12626,7 @@
       </c>
       <c r="M13" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-02-From-Rules-to-Agents.md</t>
+          <t>Modules/00-Foundations/00-04-From-Rules-to-Agents.md</t>
         </is>
       </c>
       <c r="N13" s="11" t="inlineStr">
@@ -12644,7 +12644,7 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>00-03</t>
+          <t>00-06</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
@@ -12695,7 +12695,7 @@
       </c>
       <c r="M14" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-03-BankCo-Decision-Support-Warmup.md</t>
+          <t>Modules/00-Foundations/00-06-BankCo-Decision-Support-Warmup.md</t>
         </is>
       </c>
       <c r="N14" s="11" t="inlineStr">
@@ -12713,7 +12713,7 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>00-03</t>
+          <t>00-06</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="M15" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-03-BankCo-Decision-Support-Warmup.md</t>
+          <t>Modules/00-Foundations/00-06-BankCo-Decision-Support-Warmup.md</t>
         </is>
       </c>
       <c r="N15" s="11" t="inlineStr">
@@ -12782,7 +12782,7 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>00-03</t>
+          <t>00-06</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
@@ -12833,7 +12833,7 @@
       </c>
       <c r="M16" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-03-BankCo-Decision-Support-Warmup.md</t>
+          <t>Modules/00-Foundations/00-06-BankCo-Decision-Support-Warmup.md</t>
         </is>
       </c>
       <c r="N16" s="11" t="inlineStr">
@@ -12851,7 +12851,7 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>00-03</t>
+          <t>00-06</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
@@ -12902,7 +12902,7 @@
       </c>
       <c r="M17" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-03-BankCo-Decision-Support-Warmup.md</t>
+          <t>Modules/00-Foundations/00-06-BankCo-Decision-Support-Warmup.md</t>
         </is>
       </c>
       <c r="N17" s="11" t="inlineStr">
@@ -12920,7 +12920,7 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>00-03</t>
+          <t>00-06</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
@@ -12971,7 +12971,7 @@
       </c>
       <c r="M18" s="11" t="inlineStr">
         <is>
-          <t>Modules/00-Foundations/00-03-BankCo-Decision-Support-Warmup.md</t>
+          <t>Modules/00-Foundations/00-06-BankCo-Decision-Support-Warmup.md</t>
         </is>
       </c>
       <c r="N18" s="11" t="inlineStr">
@@ -31989,7 +31989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -32320,12 +32320,12 @@
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>Principal-Staff-Interview-Guide</t>
+          <t>India-AI-Career-Learning-Plan</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Principal / Staff AI Interview Guide</t>
+          <t>India AI Career Learning Plan — From Basic Programming, Zero AI</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -32358,20 +32358,71 @@
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>Career/India-AI-Career-Learning-Plan.md</t>
+        </is>
+      </c>
+      <c r="K7" s="11" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Principal-Staff-Interview-Guide</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Principal / Staff AI Interview Guide</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Leadership &amp; Career</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Career</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>IC+EM</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>00-01, 08-03, 11-01</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J7" s="11" t="inlineStr">
+      <c r="J8" s="11" t="inlineStr">
         <is>
           <t>Career/Principal-Staff-Interview-Guide.md</t>
         </is>
       </c>
-      <c r="K7" s="11" t="inlineStr"/>
+      <c r="K8" s="11" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K7"/>
+  <autoFilter ref="A1:K8"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Done,Interview-ready"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Align module IDs with Track D study order across series
Renumber Module 01 (providers before inference), Module 03
(LangGraph before patterns), and Module 10 (cost before Redis/Kafka)
so ascending IDs match the primary course path. Sync COURSE, Study Plan,
India plan, TOC, tracker, and fix broken diagram/link refs.

Co-authored-by: Rahul Chaudhari <rcrahul4@gmail.com>
</commit_message>
<xml_diff>
--- a/Tracker/GenAI-Masterclass-Tracker.xlsx
+++ b/Tracker/GenAI-Masterclass-Tracker.xlsx
@@ -860,7 +860,7 @@
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>00-01, 00-02, 00-03, 00-05</t>
+          <t>00-01, 00-02, 00-03</t>
         </is>
       </c>
       <c r="E2" s="11" t="inlineStr">
@@ -883,10 +883,10 @@
         </is>
       </c>
       <c r="J2" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K2" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-05",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-05",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-01",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-02",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-03",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L2" s="13">
@@ -901,7 +901,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>Foundations — Rules / BankCo</t>
+          <t>Foundations — rules + math + BankCo</t>
         </is>
       </c>
       <c r="C3" s="11" t="inlineStr">
@@ -911,12 +911,12 @@
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>00-04, 00-06</t>
+          <t>00-04, 00-05, 00-06</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>When-not-to-agent memo · BankCo rules</t>
+          <t>When-not-to-agent · cosine · BankCo</t>
         </is>
       </c>
       <c r="F3" s="11" t="inlineStr">
@@ -934,10 +934,10 @@
         </is>
       </c>
       <c r="J3" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K3" s="11">
-        <f>COUNTIFS(Modules!$A:$A,"00-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-04",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-06",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-06",Modules!$I:$I,"Interview-ready")</f>
+        <f>COUNTIFS(Modules!$A:$A,"00-04",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-04",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-05",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-05",Modules!$I:$I,"Interview-ready")+COUNTIFS(Modules!$A:$A,"00-06",Modules!$I:$I,"Done")+COUNTIFS(Modules!$A:$A,"00-06",Modules!$I:$I,"Interview-ready")</f>
         <v/>
       </c>
       <c r="L3" s="13">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
-          <t>01-04, 01-05</t>
+          <t>01-03, 01-04</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr"/>
@@ -3684,7 +3684,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>02-02, 03-03</t>
+          <t>02-02, 03-04</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr"/>
@@ -3798,7 +3798,7 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>03-04</t>
+          <t>03-03</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr"/>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>10-01, 10-02, 10-04</t>
+          <t>10-01, 10-02, 10-03</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr"/>
@@ -4490,7 +4490,7 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>05-01, 10-04</t>
+          <t>05-01, 10-03</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>03-04, 08-01</t>
+          <t>03-03, 08-01</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -5327,7 +5327,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6">
         <f>IFERROR(VLOOKUP(A6,Modules!$A:$I,9,FALSE),"")</f>
@@ -5446,7 +5446,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>01-03 — Inference Serving with vLLM, Ollama &amp; Quantization</t>
+          <t>01-03 — Provider SDKs: OpenAI, Claude, Gemini &amp; DeepSeek</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>01-05 — Provider SDKs: OpenAI, Claude, Gemini &amp; DeepSeek</t>
+          <t>01-05 — Inference Serving with vLLM, Ollama &amp; Quantization</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -5670,7 +5670,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>03-03 — Agentic Design Patterns: Routing, Reflection, ReAct &amp; More</t>
+          <t>03-03 — LangGraph Production Agents: State, Memory, HITL &amp; Deployment</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>03-04 — LangGraph Production Agents: State, Memory, HITL &amp; Deployment</t>
+          <t>03-04 — Agentic Design Patterns: Routing, Reflection, ReAct &amp; More</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>10-03 — Redis, Kafka &amp; Ray: Async Infrastructure for AI Platforms</t>
+          <t>10-03 — Cost &amp; Latency Optimization for LLM Systems</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -6438,7 +6438,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>10-04 — Cost &amp; Latency Optimization for LLM Systems</t>
+          <t>10-04 — Redis, Kafka &amp; Ray: Async Infrastructure for AI Platforms</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -8528,7 +8528,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
@@ -8799,7 +8799,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>01-03 — Inference Serving with vLLM, Ollama &amp; Quantization</t>
+          <t>01-03 — Provider SDKs: OpenAI, Claude, Gemini &amp; DeepSeek</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -8824,7 +8824,7 @@
         </is>
       </c>
       <c r="H10" s="11" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
@@ -8850,7 +8850,7 @@
       <c r="N10" s="11" t="inlineStr"/>
       <c r="O10" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-03-Inference-Serving-vLLM.md</t>
+          <t>Modules/01-LLM-Engineering/01-03-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
         </is>
       </c>
       <c r="P10" s="12">
@@ -8943,7 +8943,7 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>01-05 — Provider SDKs: OpenAI, Claude, Gemini &amp; DeepSeek</t>
+          <t>01-05 — Inference Serving with vLLM, Ollama &amp; Quantization</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -8968,7 +8968,7 @@
         </is>
       </c>
       <c r="H12" s="11" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
@@ -8994,7 +8994,7 @@
       <c r="N12" s="11" t="inlineStr"/>
       <c r="O12" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-05-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
+          <t>Modules/01-LLM-Engineering/01-05-Inference-Serving-vLLM.md</t>
         </is>
       </c>
       <c r="P12" s="12">
@@ -9303,7 +9303,7 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>03-03 — Agentic Design Patterns: Routing, Reflection, ReAct &amp; More</t>
+          <t>03-03 — LangGraph Production Agents: State, Memory, HITL &amp; Deployment</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
@@ -9328,7 +9328,7 @@
         </is>
       </c>
       <c r="H17" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
@@ -9354,7 +9354,7 @@
       <c r="N17" s="11" t="inlineStr"/>
       <c r="O17" s="11" t="inlineStr">
         <is>
-          <t>Modules/03-Agentic-Fundamentals/03-03-Agentic-Design-Patterns.md</t>
+          <t>Modules/03-Agentic-Fundamentals/03-03-LangGraph-Production-Agents.md</t>
         </is>
       </c>
       <c r="P17" s="12">
@@ -9375,7 +9375,7 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>03-04 — LangGraph Production Agents: State, Memory, HITL &amp; Deployment</t>
+          <t>03-04 — Agentic Design Patterns: Routing, Reflection, ReAct &amp; More</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
@@ -9400,7 +9400,7 @@
         </is>
       </c>
       <c r="H18" s="11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
@@ -9426,7 +9426,7 @@
       <c r="N18" s="11" t="inlineStr"/>
       <c r="O18" s="11" t="inlineStr">
         <is>
-          <t>Modules/03-Agentic-Fundamentals/03-04-LangGraph-Production-Agents.md</t>
+          <t>Modules/03-Agentic-Fundamentals/03-04-Agentic-Design-Patterns.md</t>
         </is>
       </c>
       <c r="P18" s="12">
@@ -10959,7 +10959,7 @@
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>10-03 — Redis, Kafka &amp; Ray: Async Infrastructure for AI Platforms</t>
+          <t>10-03 — Cost &amp; Latency Optimization for LLM Systems</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
@@ -11010,7 +11010,7 @@
       <c r="N40" s="11" t="inlineStr"/>
       <c r="O40" s="11" t="inlineStr">
         <is>
-          <t>Modules/10-Production-Infrastructure/10-03-Redis-Kafka-Ray.md</t>
+          <t>Modules/10-Production-Infrastructure/10-03-Cost-Latency-Optimization.md</t>
         </is>
       </c>
       <c r="P40" s="12">
@@ -11031,7 +11031,7 @@
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>10-04 — Cost &amp; Latency Optimization for LLM Systems</t>
+          <t>10-04 — Redis, Kafka &amp; Ray: Async Infrastructure for AI Platforms</t>
         </is>
       </c>
       <c r="C41" s="11" t="inlineStr">
@@ -11082,7 +11082,7 @@
       <c r="N41" s="11" t="inlineStr"/>
       <c r="O41" s="11" t="inlineStr">
         <is>
-          <t>Modules/10-Production-Infrastructure/10-04-Cost-Latency-Optimization.md</t>
+          <t>Modules/10-Production-Infrastructure/10-04-Redis-Kafka-Ray.md</t>
         </is>
       </c>
       <c r="P41" s="12">
@@ -13899,12 +13899,12 @@
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>vLLM Documentation</t>
+          <t>OpenAI API Documentation</t>
         </is>
       </c>
       <c r="F32" s="12" t="inlineStr">
         <is>
-          <t>https://docs.vllm.ai/en/latest/</t>
+          <t>https://developers.openai.com/api/docs/</t>
         </is>
       </c>
       <c r="G32" s="12">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Intro</t>
         </is>
       </c>
       <c r="J32" s="11" t="inlineStr">
@@ -13927,17 +13927,17 @@
       </c>
       <c r="K32" s="11" t="inlineStr">
         <is>
-          <t>Official serving flags, APIs, schedulers</t>
+          <t>Canonical Responses + tools reference</t>
         </is>
       </c>
       <c r="L32" s="11" t="inlineStr">
         <is>
-          <t>Installation; OpenAI server; optimization</t>
+          <t>Responses API; structured outputs; streaming</t>
         </is>
       </c>
       <c r="M32" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-03-Inference-Serving-vLLM.md</t>
+          <t>Modules/01-LLM-Engineering/01-03-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
         </is>
       </c>
       <c r="N32" s="11" t="inlineStr">
@@ -13968,12 +13968,12 @@
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>vLLM GitHub</t>
+          <t>OpenAI Python SDK</t>
         </is>
       </c>
       <c r="F33" s="12" t="inlineStr">
         <is>
-          <t>https://github.com/vllm-project/vllm</t>
+          <t>https://github.com/openai/openai-python</t>
         </is>
       </c>
       <c r="G33" s="12">
@@ -13986,7 +13986,7 @@
       </c>
       <c r="I33" s="11" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Intro</t>
         </is>
       </c>
       <c r="J33" s="11" t="inlineStr">
@@ -13996,17 +13996,17 @@
       </c>
       <c r="K33" s="11" t="inlineStr">
         <is>
-          <t>Issue tracker, release notes, examples</t>
+          <t>`responses.parse`, streaming helpers</t>
         </is>
       </c>
       <c r="L33" s="11" t="inlineStr">
         <is>
-          <t>README; performance tips</t>
+          <t>helpers.md; examples</t>
         </is>
       </c>
       <c r="M33" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-03-Inference-Serving-vLLM.md</t>
+          <t>Modules/01-LLM-Engineering/01-03-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
         </is>
       </c>
       <c r="N33" s="11" t="inlineStr">
@@ -14037,12 +14037,12 @@
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>Ollama GitHub</t>
+          <t>Anthropic API Overview</t>
         </is>
       </c>
       <c r="F34" s="12" t="inlineStr">
         <is>
-          <t>https://github.com/ollama/ollama</t>
+          <t>https://platform.claude.com/docs/en/api/overview</t>
         </is>
       </c>
       <c r="G34" s="12">
@@ -14060,22 +14060,22 @@
       </c>
       <c r="J34" s="11" t="inlineStr">
         <is>
-          <t>20 min</t>
+          <t>45 min</t>
         </is>
       </c>
       <c r="K34" s="11" t="inlineStr">
         <is>
-          <t>Local model pull/run workflow</t>
+          <t>Messages API mental model</t>
         </is>
       </c>
       <c r="L34" s="11" t="inlineStr">
         <is>
-          <t>API; modelfiles</t>
+          <t>Messages; tool use; streaming</t>
         </is>
       </c>
       <c r="M34" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-03-Inference-Serving-vLLM.md</t>
+          <t>Modules/01-LLM-Engineering/01-03-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
         </is>
       </c>
       <c r="N34" s="11" t="inlineStr">
@@ -14106,12 +14106,12 @@
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>HF Quantization</t>
+          <t>Anthropic Python SDK</t>
         </is>
       </c>
       <c r="F35" s="12" t="inlineStr">
         <is>
-          <t>https://huggingface.co/docs/transformers/en/main_classes/quantization</t>
+          <t>https://github.com/anthropics/anthropic-sdk-python</t>
         </is>
       </c>
       <c r="G35" s="12">
@@ -14124,27 +14124,27 @@
       </c>
       <c r="I35" s="11" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Intro</t>
         </is>
       </c>
       <c r="J35" s="11" t="inlineStr">
         <is>
-          <t>45 min</t>
+          <t>30 min</t>
         </is>
       </c>
       <c r="K35" s="11" t="inlineStr">
         <is>
-          <t>GPTQ/AWQ/BnB overview</t>
+          <t>Typed messages + stream context managers</t>
         </is>
       </c>
       <c r="L35" s="11" t="inlineStr">
         <is>
-          <t>Method comparison tables</t>
+          <t>README; streaming</t>
         </is>
       </c>
       <c r="M35" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-03-Inference-Serving-vLLM.md</t>
+          <t>Modules/01-LLM-Engineering/01-03-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
         </is>
       </c>
       <c r="N35" s="11" t="inlineStr">
@@ -14175,12 +14175,12 @@
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>TensorRT-LLM</t>
+          <t>Gemini API Docs</t>
         </is>
       </c>
       <c r="F36" s="12" t="inlineStr">
         <is>
-          <t>https://developer.nvidia.com/tensorrt-llm</t>
+          <t>https://ai.google.dev/gemini-api/docs</t>
         </is>
       </c>
       <c r="G36" s="12">
@@ -14193,7 +14193,7 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Intro</t>
         </is>
       </c>
       <c r="J36" s="11" t="inlineStr">
@@ -14203,17 +14203,17 @@
       </c>
       <c r="K36" s="11" t="inlineStr">
         <is>
-          <t>When compiled NVIDIA stacks win</t>
+          <t>Structured output + function calling</t>
         </is>
       </c>
       <c r="L36" s="11" t="inlineStr">
         <is>
-          <t>Quick start; perf guides</t>
+          <t>generateContent; tools; JSON schema</t>
         </is>
       </c>
       <c r="M36" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-03-Inference-Serving-vLLM.md</t>
+          <t>Modules/01-LLM-Engineering/01-03-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
         </is>
       </c>
       <c r="N36" s="11" t="inlineStr">
@@ -14244,12 +14244,12 @@
       </c>
       <c r="E37" s="11" t="inlineStr">
         <is>
-          <t>PagedAttention paper (vLLM)</t>
+          <t>Google GenAI Python SDK</t>
         </is>
       </c>
       <c r="F37" s="12" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2309.06180</t>
+          <t>https://github.com/googleapis/python-genai</t>
         </is>
       </c>
       <c r="G37" s="12">
@@ -14262,27 +14262,27 @@
       </c>
       <c r="I37" s="11" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Intro</t>
         </is>
       </c>
       <c r="J37" s="11" t="inlineStr">
         <is>
-          <t>45 min</t>
+          <t>30 min</t>
         </is>
       </c>
       <c r="K37" s="11" t="inlineStr">
         <is>
-          <t>Primary source for paging intuition</t>
+          <t>`Client`, `types`, async patterns</t>
         </is>
       </c>
       <c r="L37" s="11" t="inlineStr">
         <is>
-          <t>§3 Memory management</t>
+          <t>README; samples</t>
         </is>
       </c>
       <c r="M37" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-03-Inference-Serving-vLLM.md</t>
+          <t>Modules/01-LLM-Engineering/01-03-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
         </is>
       </c>
       <c r="N37" s="11" t="inlineStr">
@@ -14313,12 +14313,12 @@
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>Speculative Decoding</t>
+          <t>DeepSeek API Docs</t>
         </is>
       </c>
       <c r="F38" s="12" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2211.17192</t>
+          <t>https://api-docs.deepseek.com/</t>
         </is>
       </c>
       <c r="G38" s="12">
@@ -14331,7 +14331,7 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Intro</t>
         </is>
       </c>
       <c r="J38" s="11" t="inlineStr">
@@ -14341,17 +14341,17 @@
       </c>
       <c r="K38" s="11" t="inlineStr">
         <is>
-          <t>Draft/verify mental model</t>
+          <t>OpenAI-compatible cost tier</t>
         </is>
       </c>
       <c r="L38" s="11" t="inlineStr">
         <is>
-          <t>Algorithm 1</t>
+          <t>models; chat; pricing</t>
         </is>
       </c>
       <c r="M38" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-03-Inference-Serving-vLLM.md</t>
+          <t>Modules/01-LLM-Engineering/01-03-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
         </is>
       </c>
       <c r="N38" s="11" t="inlineStr">
@@ -14934,12 +14934,12 @@
       </c>
       <c r="E47" s="11" t="inlineStr">
         <is>
-          <t>OpenAI API Documentation</t>
+          <t>vLLM Documentation</t>
         </is>
       </c>
       <c r="F47" s="12" t="inlineStr">
         <is>
-          <t>https://developers.openai.com/api/docs/</t>
+          <t>https://docs.vllm.ai/en/latest/</t>
         </is>
       </c>
       <c r="G47" s="12">
@@ -14952,7 +14952,7 @@
       </c>
       <c r="I47" s="11" t="inlineStr">
         <is>
-          <t>Intro</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="J47" s="11" t="inlineStr">
@@ -14962,17 +14962,17 @@
       </c>
       <c r="K47" s="11" t="inlineStr">
         <is>
-          <t>Canonical Responses + tools reference</t>
+          <t>Official serving flags, APIs, schedulers</t>
         </is>
       </c>
       <c r="L47" s="11" t="inlineStr">
         <is>
-          <t>Responses API; structured outputs; streaming</t>
+          <t>Installation; OpenAI server; optimization</t>
         </is>
       </c>
       <c r="M47" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-05-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
+          <t>Modules/01-LLM-Engineering/01-05-Inference-Serving-vLLM.md</t>
         </is>
       </c>
       <c r="N47" s="11" t="inlineStr">
@@ -15003,12 +15003,12 @@
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>OpenAI Python SDK</t>
+          <t>vLLM GitHub</t>
         </is>
       </c>
       <c r="F48" s="12" t="inlineStr">
         <is>
-          <t>https://github.com/openai/openai-python</t>
+          <t>https://github.com/vllm-project/vllm</t>
         </is>
       </c>
       <c r="G48" s="12">
@@ -15021,7 +15021,7 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Intro</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="J48" s="11" t="inlineStr">
@@ -15031,17 +15031,17 @@
       </c>
       <c r="K48" s="11" t="inlineStr">
         <is>
-          <t>`responses.parse`, streaming helpers</t>
+          <t>Issue tracker, release notes, examples</t>
         </is>
       </c>
       <c r="L48" s="11" t="inlineStr">
         <is>
-          <t>helpers.md; examples</t>
+          <t>README; performance tips</t>
         </is>
       </c>
       <c r="M48" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-05-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
+          <t>Modules/01-LLM-Engineering/01-05-Inference-Serving-vLLM.md</t>
         </is>
       </c>
       <c r="N48" s="11" t="inlineStr">
@@ -15072,12 +15072,12 @@
       </c>
       <c r="E49" s="11" t="inlineStr">
         <is>
-          <t>Anthropic API Overview</t>
+          <t>Ollama GitHub</t>
         </is>
       </c>
       <c r="F49" s="12" t="inlineStr">
         <is>
-          <t>https://platform.claude.com/docs/en/api/overview</t>
+          <t>https://github.com/ollama/ollama</t>
         </is>
       </c>
       <c r="G49" s="12">
@@ -15095,22 +15095,22 @@
       </c>
       <c r="J49" s="11" t="inlineStr">
         <is>
-          <t>45 min</t>
+          <t>20 min</t>
         </is>
       </c>
       <c r="K49" s="11" t="inlineStr">
         <is>
-          <t>Messages API mental model</t>
+          <t>Local model pull/run workflow</t>
         </is>
       </c>
       <c r="L49" s="11" t="inlineStr">
         <is>
-          <t>Messages; tool use; streaming</t>
+          <t>API; modelfiles</t>
         </is>
       </c>
       <c r="M49" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-05-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
+          <t>Modules/01-LLM-Engineering/01-05-Inference-Serving-vLLM.md</t>
         </is>
       </c>
       <c r="N49" s="11" t="inlineStr">
@@ -15141,12 +15141,12 @@
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>Anthropic Python SDK</t>
+          <t>HF Quantization</t>
         </is>
       </c>
       <c r="F50" s="12" t="inlineStr">
         <is>
-          <t>https://github.com/anthropics/anthropic-sdk-python</t>
+          <t>https://huggingface.co/docs/transformers/en/main_classes/quantization</t>
         </is>
       </c>
       <c r="G50" s="12">
@@ -15159,27 +15159,27 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Intro</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="J50" s="11" t="inlineStr">
         <is>
-          <t>30 min</t>
+          <t>45 min</t>
         </is>
       </c>
       <c r="K50" s="11" t="inlineStr">
         <is>
-          <t>Typed messages + stream context managers</t>
+          <t>GPTQ/AWQ/BnB overview</t>
         </is>
       </c>
       <c r="L50" s="11" t="inlineStr">
         <is>
-          <t>README; streaming</t>
+          <t>Method comparison tables</t>
         </is>
       </c>
       <c r="M50" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-05-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
+          <t>Modules/01-LLM-Engineering/01-05-Inference-Serving-vLLM.md</t>
         </is>
       </c>
       <c r="N50" s="11" t="inlineStr">
@@ -15210,12 +15210,12 @@
       </c>
       <c r="E51" s="11" t="inlineStr">
         <is>
-          <t>Gemini API Docs</t>
+          <t>TensorRT-LLM</t>
         </is>
       </c>
       <c r="F51" s="12" t="inlineStr">
         <is>
-          <t>https://ai.google.dev/gemini-api/docs</t>
+          <t>https://developer.nvidia.com/tensorrt-llm</t>
         </is>
       </c>
       <c r="G51" s="12">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="I51" s="11" t="inlineStr">
         <is>
-          <t>Intro</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="J51" s="11" t="inlineStr">
@@ -15238,17 +15238,17 @@
       </c>
       <c r="K51" s="11" t="inlineStr">
         <is>
-          <t>Structured output + function calling</t>
+          <t>When compiled NVIDIA stacks win</t>
         </is>
       </c>
       <c r="L51" s="11" t="inlineStr">
         <is>
-          <t>generateContent; tools; JSON schema</t>
+          <t>Quick start; perf guides</t>
         </is>
       </c>
       <c r="M51" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-05-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
+          <t>Modules/01-LLM-Engineering/01-05-Inference-Serving-vLLM.md</t>
         </is>
       </c>
       <c r="N51" s="11" t="inlineStr">
@@ -15279,12 +15279,12 @@
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>Google GenAI Python SDK</t>
+          <t>PagedAttention paper (vLLM)</t>
         </is>
       </c>
       <c r="F52" s="12" t="inlineStr">
         <is>
-          <t>https://github.com/googleapis/python-genai</t>
+          <t>https://arxiv.org/abs/2309.06180</t>
         </is>
       </c>
       <c r="G52" s="12">
@@ -15297,27 +15297,27 @@
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Intro</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="J52" s="11" t="inlineStr">
         <is>
-          <t>30 min</t>
+          <t>45 min</t>
         </is>
       </c>
       <c r="K52" s="11" t="inlineStr">
         <is>
-          <t>`Client`, `types`, async patterns</t>
+          <t>Primary source for paging intuition</t>
         </is>
       </c>
       <c r="L52" s="11" t="inlineStr">
         <is>
-          <t>README; samples</t>
+          <t>§3 Memory management</t>
         </is>
       </c>
       <c r="M52" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-05-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
+          <t>Modules/01-LLM-Engineering/01-05-Inference-Serving-vLLM.md</t>
         </is>
       </c>
       <c r="N52" s="11" t="inlineStr">
@@ -15348,12 +15348,12 @@
       </c>
       <c r="E53" s="11" t="inlineStr">
         <is>
-          <t>DeepSeek API Docs</t>
+          <t>Speculative Decoding</t>
         </is>
       </c>
       <c r="F53" s="12" t="inlineStr">
         <is>
-          <t>https://api-docs.deepseek.com/</t>
+          <t>https://arxiv.org/abs/2211.17192</t>
         </is>
       </c>
       <c r="G53" s="12">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="I53" s="11" t="inlineStr">
         <is>
-          <t>Intro</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="J53" s="11" t="inlineStr">
@@ -15376,17 +15376,17 @@
       </c>
       <c r="K53" s="11" t="inlineStr">
         <is>
-          <t>OpenAI-compatible cost tier</t>
+          <t>Draft/verify mental model</t>
         </is>
       </c>
       <c r="L53" s="11" t="inlineStr">
         <is>
-          <t>models; chat; pricing</t>
+          <t>Algorithm 1</t>
         </is>
       </c>
       <c r="M53" s="11" t="inlineStr">
         <is>
-          <t>Modules/01-LLM-Engineering/01-05-Provider-SDKs-OpenAI-Claude-Gemini.md</t>
+          <t>Modules/01-LLM-Engineering/01-05-Inference-Serving-vLLM.md</t>
         </is>
       </c>
       <c r="N53" s="11" t="inlineStr">
@@ -17101,17 +17101,17 @@
       </c>
       <c r="K78" s="11" t="inlineStr">
         <is>
-          <t>Persistence + HITL foundation for patterns</t>
+          <t>Runtime mental model</t>
         </is>
       </c>
       <c r="L78" s="11" t="inlineStr">
         <is>
-          <t>Benefits; state; checkpointers</t>
+          <t>Persistence; compile</t>
         </is>
       </c>
       <c r="M78" s="11" t="inlineStr">
         <is>
-          <t>Modules/03-Agentic-Fundamentals/03-03-Agentic-Design-Patterns.md</t>
+          <t>Modules/03-Agentic-Fundamentals/03-03-LangGraph-Production-Agents.md</t>
         </is>
       </c>
       <c r="N78" s="11" t="inlineStr">
@@ -17142,7 +17142,7 @@
       </c>
       <c r="E79" s="11" t="inlineStr">
         <is>
-          <t>LangGraph Human-in-the-Loop</t>
+          <t>Human-in-the-Loop</t>
         </is>
       </c>
       <c r="F79" s="12" t="inlineStr">
@@ -17165,22 +17165,22 @@
       </c>
       <c r="J79" s="11" t="inlineStr">
         <is>
-          <t>30 min</t>
+          <t>35 min</t>
         </is>
       </c>
       <c r="K79" s="11" t="inlineStr">
         <is>
-          <t>Interrupt/resume semantics</t>
+          <t>Interrupt/resume</t>
         </is>
       </c>
       <c r="L79" s="11" t="inlineStr">
         <is>
-          <t>Breakpoints; approve/edit</t>
+          <t>Breakpoints; Command</t>
         </is>
       </c>
       <c r="M79" s="11" t="inlineStr">
         <is>
-          <t>Modules/03-Agentic-Fundamentals/03-03-Agentic-Design-Patterns.md</t>
+          <t>Modules/03-Agentic-Fundamentals/03-03-LangGraph-Production-Agents.md</t>
         </is>
       </c>
       <c r="N79" s="11" t="inlineStr">
@@ -17211,12 +17211,12 @@
       </c>
       <c r="E80" s="11" t="inlineStr">
         <is>
-          <t>ReAct Paper</t>
+          <t>Streaming</t>
         </is>
       </c>
       <c r="F80" s="12" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2210.03629</t>
+          <t>https://langchain-ai.github.io/langgraph/concepts/streaming/</t>
         </is>
       </c>
       <c r="G80" s="12">
@@ -17234,22 +17234,22 @@
       </c>
       <c r="J80" s="11" t="inlineStr">
         <is>
-          <t>45 min</t>
+          <t>30 min</t>
         </is>
       </c>
       <c r="K80" s="11" t="inlineStr">
         <is>
-          <t>Original Think-Act-Observe</t>
+          <t>UX + debugging</t>
         </is>
       </c>
       <c r="L80" s="11" t="inlineStr">
         <is>
-          <t>Examples; synergy</t>
+          <t>stream_mode options</t>
         </is>
       </c>
       <c r="M80" s="11" t="inlineStr">
         <is>
-          <t>Modules/03-Agentic-Fundamentals/03-03-Agentic-Design-Patterns.md</t>
+          <t>Modules/03-Agentic-Fundamentals/03-03-LangGraph-Production-Agents.md</t>
         </is>
       </c>
       <c r="N80" s="11" t="inlineStr">
@@ -17280,12 +17280,12 @@
       </c>
       <c r="E81" s="11" t="inlineStr">
         <is>
-          <t>LangSmith</t>
+          <t>Multi-Agent</t>
         </is>
       </c>
       <c r="F81" s="12" t="inlineStr">
         <is>
-          <t>https://docs.langchain.com/langsmith/home</t>
+          <t>https://langchain-ai.github.io/langgraph/concepts/multi_agent/</t>
         </is>
       </c>
       <c r="G81" s="12">
@@ -17298,27 +17298,27 @@
       </c>
       <c r="I81" s="11" t="inlineStr">
         <is>
-          <t>Intro</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="J81" s="11" t="inlineStr">
         <is>
-          <t>20 min</t>
+          <t>40 min</t>
         </is>
       </c>
       <c r="K81" s="11" t="inlineStr">
         <is>
-          <t>Trace routes and tool loops</t>
+          <t>When to split graphs</t>
         </is>
       </c>
       <c r="L81" s="11" t="inlineStr">
         <is>
-          <t>Projects; runs; feedback</t>
+          <t>Supervisor; handoffs</t>
         </is>
       </c>
       <c r="M81" s="11" t="inlineStr">
         <is>
-          <t>Modules/03-Agentic-Fundamentals/03-03-Agentic-Design-Patterns.md</t>
+          <t>Modules/03-Agentic-Fundamentals/03-03-LangGraph-Production-Agents.md</t>
         </is>
       </c>
       <c r="N81" s="11" t="inlineStr">
@@ -17336,7 +17336,7 @@
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
-          <t>03-04</t>
+          <t>03-03</t>
         </is>
       </c>
       <c r="C82" s="11" t="inlineStr">
@@ -17345,16 +17345,16 @@
         </is>
       </c>
       <c r="D82" s="11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E82" s="11" t="inlineStr">
         <is>
-          <t>LangGraph High Level</t>
+          <t>LangSmith</t>
         </is>
       </c>
       <c r="F82" s="12" t="inlineStr">
         <is>
-          <t>https://langchain-ai.github.io/langgraph/concepts/high_level/</t>
+          <t>https://docs.langchain.com/langsmith/home</t>
         </is>
       </c>
       <c r="G82" s="12">
@@ -17377,17 +17377,17 @@
       </c>
       <c r="K82" s="11" t="inlineStr">
         <is>
-          <t>Runtime mental model</t>
+          <t>Trace production graphs</t>
         </is>
       </c>
       <c r="L82" s="11" t="inlineStr">
         <is>
-          <t>Persistence; compile</t>
+          <t>Projects; evaluations</t>
         </is>
       </c>
       <c r="M82" s="11" t="inlineStr">
         <is>
-          <t>Modules/03-Agentic-Fundamentals/03-04-LangGraph-Production-Agents.md</t>
+          <t>Modules/03-Agentic-Fundamentals/03-03-LangGraph-Production-Agents.md</t>
         </is>
       </c>
       <c r="N82" s="11" t="inlineStr">
@@ -17414,16 +17414,16 @@
         </is>
       </c>
       <c r="D83" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E83" s="11" t="inlineStr">
         <is>
-          <t>Human-in-the-Loop</t>
+          <t>LangGraph High Level</t>
         </is>
       </c>
       <c r="F83" s="12" t="inlineStr">
         <is>
-          <t>https://langchain-ai.github.io/langgraph/concepts/human_in_the_loop/</t>
+          <t>https://langchain-ai.github.io/langgraph/concepts/high_level/</t>
         </is>
       </c>
       <c r="G83" s="12">
@@ -17436,27 +17436,27 @@
       </c>
       <c r="I83" s="11" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Intro</t>
         </is>
       </c>
       <c r="J83" s="11" t="inlineStr">
         <is>
-          <t>35 min</t>
+          <t>25 min</t>
         </is>
       </c>
       <c r="K83" s="11" t="inlineStr">
         <is>
-          <t>Interrupt/resume</t>
+          <t>Persistence + HITL foundation for patterns</t>
         </is>
       </c>
       <c r="L83" s="11" t="inlineStr">
         <is>
-          <t>Breakpoints; Command</t>
+          <t>Benefits; state; checkpointers</t>
         </is>
       </c>
       <c r="M83" s="11" t="inlineStr">
         <is>
-          <t>Modules/03-Agentic-Fundamentals/03-04-LangGraph-Production-Agents.md</t>
+          <t>Modules/03-Agentic-Fundamentals/03-04-Agentic-Design-Patterns.md</t>
         </is>
       </c>
       <c r="N83" s="11" t="inlineStr">
@@ -17483,16 +17483,16 @@
         </is>
       </c>
       <c r="D84" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E84" s="11" t="inlineStr">
         <is>
-          <t>Streaming</t>
+          <t>LangGraph Human-in-the-Loop</t>
         </is>
       </c>
       <c r="F84" s="12" t="inlineStr">
         <is>
-          <t>https://langchain-ai.github.io/langgraph/concepts/streaming/</t>
+          <t>https://langchain-ai.github.io/langgraph/concepts/human_in_the_loop/</t>
         </is>
       </c>
       <c r="G84" s="12">
@@ -17515,17 +17515,17 @@
       </c>
       <c r="K84" s="11" t="inlineStr">
         <is>
-          <t>UX + debugging</t>
+          <t>Interrupt/resume semantics</t>
         </is>
       </c>
       <c r="L84" s="11" t="inlineStr">
         <is>
-          <t>stream_mode options</t>
+          <t>Breakpoints; approve/edit</t>
         </is>
       </c>
       <c r="M84" s="11" t="inlineStr">
         <is>
-          <t>Modules/03-Agentic-Fundamentals/03-04-LangGraph-Production-Agents.md</t>
+          <t>Modules/03-Agentic-Fundamentals/03-04-Agentic-Design-Patterns.md</t>
         </is>
       </c>
       <c r="N84" s="11" t="inlineStr">
@@ -17552,16 +17552,16 @@
         </is>
       </c>
       <c r="D85" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E85" s="11" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>ReAct Paper</t>
         </is>
       </c>
       <c r="F85" s="12" t="inlineStr">
         <is>
-          <t>https://langchain-ai.github.io/langgraph/concepts/multi_agent/</t>
+          <t>https://arxiv.org/abs/2210.03629</t>
         </is>
       </c>
       <c r="G85" s="12">
@@ -17574,27 +17574,27 @@
       </c>
       <c r="I85" s="11" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="J85" s="11" t="inlineStr">
         <is>
-          <t>40 min</t>
+          <t>45 min</t>
         </is>
       </c>
       <c r="K85" s="11" t="inlineStr">
         <is>
-          <t>When to split graphs</t>
+          <t>Original Think-Act-Observe</t>
         </is>
       </c>
       <c r="L85" s="11" t="inlineStr">
         <is>
-          <t>Supervisor; handoffs</t>
+          <t>Examples; synergy</t>
         </is>
       </c>
       <c r="M85" s="11" t="inlineStr">
         <is>
-          <t>Modules/03-Agentic-Fundamentals/03-04-LangGraph-Production-Agents.md</t>
+          <t>Modules/03-Agentic-Fundamentals/03-04-Agentic-Design-Patterns.md</t>
         </is>
       </c>
       <c r="N85" s="11" t="inlineStr">
@@ -17621,7 +17621,7 @@
         </is>
       </c>
       <c r="D86" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E86" s="11" t="inlineStr">
         <is>
@@ -17648,22 +17648,22 @@
       </c>
       <c r="J86" s="11" t="inlineStr">
         <is>
-          <t>25 min</t>
+          <t>20 min</t>
         </is>
       </c>
       <c r="K86" s="11" t="inlineStr">
         <is>
-          <t>Trace production graphs</t>
+          <t>Trace routes and tool loops</t>
         </is>
       </c>
       <c r="L86" s="11" t="inlineStr">
         <is>
-          <t>Projects; evaluations</t>
+          <t>Projects; runs; feedback</t>
         </is>
       </c>
       <c r="M86" s="11" t="inlineStr">
         <is>
-          <t>Modules/03-Agentic-Fundamentals/03-04-LangGraph-Production-Agents.md</t>
+          <t>Modules/03-Agentic-Fundamentals/03-04-Agentic-Design-Patterns.md</t>
         </is>
       </c>
       <c r="N86" s="11" t="inlineStr">
@@ -24965,12 +24965,12 @@
       </c>
       <c r="E194" s="11" t="inlineStr">
         <is>
-          <t>Redis Documentation</t>
+          <t>vLLM Documentation</t>
         </is>
       </c>
       <c r="F194" s="12" t="inlineStr">
         <is>
-          <t>https://redis.io/docs/latest/</t>
+          <t>https://docs.vllm.ai/en/latest/</t>
         </is>
       </c>
       <c r="G194" s="12">
@@ -24983,27 +24983,27 @@
       </c>
       <c r="I194" s="11" t="inlineStr">
         <is>
-          <t>Intro</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="J194" s="11" t="inlineStr">
         <is>
-          <t>45 min</t>
+          <t>30 min</t>
         </is>
       </c>
       <c r="K194" s="11" t="inlineStr">
         <is>
-          <t>Commands &amp; patterns</t>
+          <t>Throughput knobs</t>
         </is>
       </c>
       <c r="L194" s="11" t="inlineStr">
         <is>
-          <t>Data types; TTL</t>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="M194" s="11" t="inlineStr">
         <is>
-          <t>Modules/10-Production-Infrastructure/10-03-Redis-Kafka-Ray.md</t>
+          <t>Modules/10-Production-Infrastructure/10-03-Cost-Latency-Optimization.md</t>
         </is>
       </c>
       <c r="N194" s="11" t="inlineStr">
@@ -25034,12 +25034,12 @@
       </c>
       <c r="E195" s="11" t="inlineStr">
         <is>
-          <t>Kafka Documentation</t>
+          <t>OpenAI Pricing</t>
         </is>
       </c>
       <c r="F195" s="12" t="inlineStr">
         <is>
-          <t>https://kafka.apache.org/documentation/</t>
+          <t>https://openai.com/api/pricing/</t>
         </is>
       </c>
       <c r="G195" s="12">
@@ -25052,27 +25052,27 @@
       </c>
       <c r="I195" s="11" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Intro</t>
         </is>
       </c>
       <c r="J195" s="11" t="inlineStr">
         <is>
-          <t>60 min</t>
+          <t>15 min</t>
         </is>
       </c>
       <c r="K195" s="11" t="inlineStr">
         <is>
-          <t>Topics &amp; consumer groups</t>
+          <t>API unit costs</t>
         </is>
       </c>
       <c r="L195" s="11" t="inlineStr">
         <is>
-          <t>Introduction</t>
+          <t>Model tiers</t>
         </is>
       </c>
       <c r="M195" s="11" t="inlineStr">
         <is>
-          <t>Modules/10-Production-Infrastructure/10-03-Redis-Kafka-Ray.md</t>
+          <t>Modules/10-Production-Infrastructure/10-03-Cost-Latency-Optimization.md</t>
         </is>
       </c>
       <c r="N195" s="11" t="inlineStr">
@@ -25090,7 +25090,7 @@
       </c>
       <c r="B196" s="11" t="inlineStr">
         <is>
-          <t>10-03</t>
+          <t>10-04</t>
         </is>
       </c>
       <c r="C196" s="11" t="inlineStr">
@@ -25099,16 +25099,16 @@
         </is>
       </c>
       <c r="D196" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E196" s="11" t="inlineStr">
         <is>
-          <t>Ray Documentation</t>
+          <t>Redis Documentation</t>
         </is>
       </c>
       <c r="F196" s="12" t="inlineStr">
         <is>
-          <t>https://docs.ray.io/en/latest/</t>
+          <t>https://redis.io/docs/latest/</t>
         </is>
       </c>
       <c r="G196" s="12">
@@ -25121,27 +25121,27 @@
       </c>
       <c r="I196" s="11" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Intro</t>
         </is>
       </c>
       <c r="J196" s="11" t="inlineStr">
         <is>
-          <t>60 min</t>
+          <t>45 min</t>
         </is>
       </c>
       <c r="K196" s="11" t="inlineStr">
         <is>
-          <t>Ray Serve &amp; Train</t>
+          <t>Commands &amp; patterns</t>
         </is>
       </c>
       <c r="L196" s="11" t="inlineStr">
         <is>
-          <t>Getting started</t>
+          <t>Data types; TTL</t>
         </is>
       </c>
       <c r="M196" s="11" t="inlineStr">
         <is>
-          <t>Modules/10-Production-Infrastructure/10-03-Redis-Kafka-Ray.md</t>
+          <t>Modules/10-Production-Infrastructure/10-04-Redis-Kafka-Ray.md</t>
         </is>
       </c>
       <c r="N196" s="11" t="inlineStr">
@@ -25168,16 +25168,16 @@
         </is>
       </c>
       <c r="D197" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E197" s="11" t="inlineStr">
         <is>
-          <t>vLLM Documentation</t>
+          <t>Kafka Documentation</t>
         </is>
       </c>
       <c r="F197" s="12" t="inlineStr">
         <is>
-          <t>https://docs.vllm.ai/en/latest/</t>
+          <t>https://kafka.apache.org/documentation/</t>
         </is>
       </c>
       <c r="G197" s="12">
@@ -25195,22 +25195,22 @@
       </c>
       <c r="J197" s="11" t="inlineStr">
         <is>
-          <t>30 min</t>
+          <t>60 min</t>
         </is>
       </c>
       <c r="K197" s="11" t="inlineStr">
         <is>
-          <t>Throughput knobs</t>
+          <t>Topics &amp; consumer groups</t>
         </is>
       </c>
       <c r="L197" s="11" t="inlineStr">
         <is>
-          <t>Optimization</t>
+          <t>Introduction</t>
         </is>
       </c>
       <c r="M197" s="11" t="inlineStr">
         <is>
-          <t>Modules/10-Production-Infrastructure/10-04-Cost-Latency-Optimization.md</t>
+          <t>Modules/10-Production-Infrastructure/10-04-Redis-Kafka-Ray.md</t>
         </is>
       </c>
       <c r="N197" s="11" t="inlineStr">
@@ -25237,16 +25237,16 @@
         </is>
       </c>
       <c r="D198" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E198" s="11" t="inlineStr">
         <is>
-          <t>OpenAI Pricing</t>
+          <t>Ray Documentation</t>
         </is>
       </c>
       <c r="F198" s="12" t="inlineStr">
         <is>
-          <t>https://openai.com/api/pricing/</t>
+          <t>https://docs.ray.io/en/latest/</t>
         </is>
       </c>
       <c r="G198" s="12">
@@ -25259,27 +25259,27 @@
       </c>
       <c r="I198" s="11" t="inlineStr">
         <is>
-          <t>Intro</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="J198" s="11" t="inlineStr">
         <is>
-          <t>15 min</t>
+          <t>60 min</t>
         </is>
       </c>
       <c r="K198" s="11" t="inlineStr">
         <is>
-          <t>API unit costs</t>
+          <t>Ray Serve &amp; Train</t>
         </is>
       </c>
       <c r="L198" s="11" t="inlineStr">
         <is>
-          <t>Model tiers</t>
+          <t>Getting started</t>
         </is>
       </c>
       <c r="M198" s="11" t="inlineStr">
         <is>
-          <t>Modules/10-Production-Infrastructure/10-04-Cost-Latency-Optimization.md</t>
+          <t>Modules/10-Production-Infrastructure/10-04-Redis-Kafka-Ray.md</t>
         </is>
       </c>
       <c r="N198" s="11" t="inlineStr">
@@ -31137,7 +31137,7 @@
       <c r="H2" s="11" t="inlineStr"/>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>03-01, 03-04, 12-03</t>
+          <t>03-01, 03-03, 12-03</t>
         </is>
       </c>
       <c r="J2" s="11" t="inlineStr"/>
@@ -31203,7 +31203,7 @@
       <c r="H3" s="11" t="inlineStr"/>
       <c r="I3" s="11" t="inlineStr">
         <is>
-          <t>03-03, 04-01, 08-03</t>
+          <t>03-04, 04-01, 08-03</t>
         </is>
       </c>
       <c r="J3" s="11" t="inlineStr"/>
@@ -31335,7 +31335,7 @@
       <c r="H5" s="11" t="inlineStr"/>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>04-03, 04-04, 10-03</t>
+          <t>04-03, 04-04, 10-04</t>
         </is>
       </c>
       <c r="J5" s="11" t="inlineStr"/>
@@ -31401,7 +31401,7 @@
       <c r="H6" s="11" t="inlineStr"/>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>06-01, 10-04, 08-02</t>
+          <t>06-01, 10-03, 08-02</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr"/>
@@ -31533,7 +31533,7 @@
       <c r="H8" s="11" t="inlineStr"/>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>01-05, 03-02, 07-01, 11-02</t>
+          <t>01-03, 03-02, 07-01, 11-02</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr"/>
@@ -31599,7 +31599,7 @@
       <c r="H9" s="11" t="inlineStr"/>
       <c r="I9" s="11" t="inlineStr">
         <is>
-          <t>03-04, 04-01, 12-03</t>
+          <t>03-03, 04-01, 12-03</t>
         </is>
       </c>
       <c r="J9" s="11" t="inlineStr"/>
@@ -31665,7 +31665,7 @@
       <c r="H10" s="11" t="inlineStr"/>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>01-03, 02-02, 10-04</t>
+          <t>01-05, 02-02, 10-03</t>
         </is>
       </c>
       <c r="J10" s="11" t="inlineStr"/>

</xml_diff>